<commit_message>
+ results for special benchmarking
</commit_message>
<xml_diff>
--- a/benchmarking/search_for_best_combination/results_basic.xlsx
+++ b/benchmarking/search_for_best_combination/results_basic.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11210"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/deborahdore/Documents/political-debates-graph-analysis/benchmarking/search_for_best_combination/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0D21CB4-5EE7-8B4E-BE05-9F7B72CB52CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6A72004-59BA-5642-BFD9-989F351B320B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4280" yWindow="500" windowWidth="46920" windowHeight="26600" xr2:uid="{E2EDC037-19C4-FE46-A599-BB595128A04F}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="51200" windowHeight="28800" activeTab="2" xr2:uid="{E2EDC037-19C4-FE46-A599-BB595128A04F}"/>
   </bookViews>
   <sheets>
     <sheet name="Results BASIC" sheetId="1" r:id="rId1"/>
     <sheet name="Results SPECIAL" sheetId="5" r:id="rId2"/>
-    <sheet name="trial 1" sheetId="2" r:id="rId3"/>
+    <sheet name="Results PRETRAINED" sheetId="6" r:id="rId3"/>
+    <sheet name="trial 1" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1108" uniqueCount="567">
   <si>
     <t>MODEL'S TYPE</t>
   </si>
@@ -1364,9 +1365,6 @@
     <t>TRIPLE CLASSIFICATION F1-MACRO</t>
   </si>
   <si>
-    <t>RELATION CLASSIFICATION HITS@1</t>
-  </si>
-  <si>
     <t>0.1553265707</t>
   </si>
   <si>
@@ -1410,13 +1408,502 @@
   </si>
   <si>
     <t>0.5795910651</t>
+  </si>
+  <si>
+    <t>0.2933740192</t>
+  </si>
+  <si>
+    <t>0.2942062297</t>
+  </si>
+  <si>
+    <t>0.0105413331</t>
+  </si>
+  <si>
+    <t>0.5956281515</t>
+  </si>
+  <si>
+    <t>0.3391163611</t>
+  </si>
+  <si>
+    <t>0.054569232</t>
+  </si>
+  <si>
+    <t>0.007212491</t>
+  </si>
+  <si>
+    <t>0.1673931997</t>
+  </si>
+  <si>
+    <t>0.3931609777</t>
+  </si>
+  <si>
+    <t>0.2490125493</t>
+  </si>
+  <si>
+    <t>0.3218276928</t>
+  </si>
+  <si>
+    <t>0.2502179599</t>
+  </si>
+  <si>
+    <t>0.4032654355</t>
+  </si>
+  <si>
+    <t>0.4791558137</t>
+  </si>
+  <si>
+    <t>0.4535694682</t>
+  </si>
+  <si>
+    <t>0.0002280632</t>
+  </si>
+  <si>
+    <t>0.0066708478</t>
+  </si>
+  <si>
+    <t>0.000285079</t>
+  </si>
+  <si>
+    <t>0.6088653148</t>
+  </si>
+  <si>
+    <t>0.2564452529</t>
+  </si>
+  <si>
+    <t>0.4661326187</t>
+  </si>
+  <si>
+    <t>0.0280232624</t>
+  </si>
+  <si>
+    <t>0.6831062204</t>
+  </si>
+  <si>
+    <t>0.910646471</t>
+  </si>
+  <si>
+    <t>0.6919275876</t>
+  </si>
+  <si>
+    <t>0.480671646</t>
+  </si>
+  <si>
+    <t>0.0175323564</t>
+  </si>
+  <si>
+    <t>0.7417754718</t>
+  </si>
+  <si>
+    <t>0.9276287858</t>
+  </si>
+  <si>
+    <t>0.5094550589</t>
+  </si>
+  <si>
+    <t>0.0170661553</t>
+  </si>
+  <si>
+    <t>0.2404602109</t>
+  </si>
+  <si>
+    <t>0.5804005453</t>
+  </si>
+  <si>
+    <t>0.465284563</t>
+  </si>
+  <si>
+    <t>0.0310642378</t>
+  </si>
+  <si>
+    <t>0.0023969319</t>
+  </si>
+  <si>
+    <t>0.3355704698</t>
+  </si>
+  <si>
+    <t>0.5299550926</t>
+  </si>
+  <si>
+    <t>0.5122215883</t>
+  </si>
+  <si>
+    <t>0.0723873442</t>
+  </si>
+  <si>
+    <t>0.3039309684</t>
+  </si>
+  <si>
+    <t>0.4956840512</t>
+  </si>
+  <si>
+    <t>RELATION CLASSIFICATION F1-MACRO</t>
+  </si>
+  <si>
+    <t>RELATION CLASSIFICATION  F1-MACRO</t>
+  </si>
+  <si>
+    <t>0.4994655866</t>
+  </si>
+  <si>
+    <t>0.0166698601</t>
+  </si>
+  <si>
+    <t>0.0008622341</t>
+  </si>
+  <si>
+    <t>0.3402950757</t>
+  </si>
+  <si>
+    <t>0.5492511854</t>
+  </si>
+  <si>
+    <t>0.478671288</t>
+  </si>
+  <si>
+    <t>0.0433033148</t>
+  </si>
+  <si>
+    <t>0.0017244683</t>
+  </si>
+  <si>
+    <t>0.2019543974</t>
+  </si>
+  <si>
+    <t>0.4589542718</t>
+  </si>
+  <si>
+    <t>0.4385853739</t>
+  </si>
+  <si>
+    <t>0.0453151945</t>
+  </si>
+  <si>
+    <t>0.0023950949</t>
+  </si>
+  <si>
+    <t>0.4433799578</t>
+  </si>
+  <si>
+    <t>0.5099332866</t>
+  </si>
+  <si>
+    <t>0.5044039011</t>
+  </si>
+  <si>
+    <t>0.0002876318</t>
+  </si>
+  <si>
+    <t>0.001725791</t>
+  </si>
+  <si>
+    <t>0.0418024928</t>
+  </si>
+  <si>
+    <t>0.4571895079</t>
+  </si>
+  <si>
+    <t>0.4699553022</t>
+  </si>
+  <si>
+    <t>0.00105465</t>
+  </si>
+  <si>
+    <t>0.0032598274</t>
+  </si>
+  <si>
+    <t>0.3911792905</t>
+  </si>
+  <si>
+    <t>0.5119392176</t>
+  </si>
+  <si>
+    <t>0.4891058816</t>
+  </si>
+  <si>
+    <t>0.0708533078</t>
+  </si>
+  <si>
+    <t>0.0011505273</t>
+  </si>
+  <si>
+    <t>0.4381591563</t>
+  </si>
+  <si>
+    <t>0.5397296813</t>
+  </si>
+  <si>
+    <t>0.490206793</t>
+  </si>
+  <si>
+    <t>0.0007670182</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1702780441 </t>
+  </si>
+  <si>
+    <t>0.4649348343</t>
+  </si>
+  <si>
+    <t>0.4712773825</t>
+  </si>
+  <si>
+    <t>0.0821668265</t>
+  </si>
+  <si>
+    <t>0.0000958773</t>
+  </si>
+  <si>
+    <t>0.4207094919</t>
+  </si>
+  <si>
+    <t>0.8129029676</t>
+  </si>
+  <si>
+    <t>0.4417925586</t>
+  </si>
+  <si>
+    <t>0.0566634708</t>
+  </si>
+  <si>
+    <t>0.0092042186</t>
+  </si>
+  <si>
+    <t>0.421093001</t>
+  </si>
+  <si>
+    <t>0.8192002356</t>
+  </si>
+  <si>
+    <t>0.4449338285</t>
+  </si>
+  <si>
+    <t>0.474982833</t>
+  </si>
+  <si>
+    <t>0.4543683036</t>
+  </si>
+  <si>
+    <t>0.0687440077</t>
+  </si>
+  <si>
+    <t>0.0061361457</t>
+  </si>
+  <si>
+    <t>0.4496644295</t>
+  </si>
+  <si>
+    <t>0.7975278513</t>
+  </si>
+  <si>
+    <t>0.4432182786</t>
+  </si>
+  <si>
+    <t>0.0473633749</t>
+  </si>
+  <si>
+    <t>0.5944391179</t>
+  </si>
+  <si>
+    <t>0.7450181117</t>
+  </si>
+  <si>
+    <t>0.4971688589</t>
+  </si>
+  <si>
+    <t>0.1474592522</t>
+  </si>
+  <si>
+    <t>0.4981744002</t>
+  </si>
+  <si>
+    <t>0.4820336929</t>
+  </si>
+  <si>
+    <t>0.0029721956</t>
+  </si>
+  <si>
+    <t>0.0056567594</t>
+  </si>
+  <si>
+    <t>0.2316395014</t>
+  </si>
+  <si>
+    <t>0.550814014</t>
+  </si>
+  <si>
+    <t>0.4688587232</t>
+  </si>
+  <si>
+    <t>0.0262703739</t>
+  </si>
+  <si>
+    <t>0.3942473634</t>
+  </si>
+  <si>
+    <t>0.8530152464</t>
+  </si>
+  <si>
+    <t>0.433872699</t>
+  </si>
+  <si>
+    <t>0.1035474593</t>
+  </si>
+  <si>
+    <t>0.4897956212</t>
+  </si>
+  <si>
+    <t>0.4776966775</t>
+  </si>
+  <si>
+    <t>0.0208053692</t>
+  </si>
+  <si>
+    <t>0.752541512</t>
+  </si>
+  <si>
+    <t>0.4026642602</t>
+  </si>
+  <si>
+    <t>0.0307766059</t>
+  </si>
+  <si>
+    <t>0.0077660594</t>
+  </si>
+  <si>
+    <t>0.5117929051</t>
+  </si>
+  <si>
+    <t>0.8680892299</t>
+  </si>
+  <si>
+    <t>0.392412305</t>
+  </si>
+  <si>
+    <t>0.0000958038</t>
+  </si>
+  <si>
+    <t>0.0010538418</t>
+  </si>
+  <si>
+    <t>0.5284434848</t>
+  </si>
+  <si>
+    <t>0.4763042531</t>
+  </si>
+  <si>
+    <t>0.0118796704</t>
+  </si>
+  <si>
+    <t>0.0143705691</t>
+  </si>
+  <si>
+    <t>0.2843456601</t>
+  </si>
+  <si>
+    <t>0.7458032071</t>
+  </si>
+  <si>
+    <t>0.4556467403</t>
+  </si>
+  <si>
+    <t>0.0413872389</t>
+  </si>
+  <si>
+    <t>0.0026825063</t>
+  </si>
+  <si>
+    <t>0.2952672926</t>
+  </si>
+  <si>
+    <t>0.712570266</t>
+  </si>
+  <si>
+    <t>0.4628218027</t>
+  </si>
+  <si>
+    <t>0.000479019</t>
+  </si>
+  <si>
+    <t>0.1576930446</t>
+  </si>
+  <si>
+    <t>0.4931564825</t>
+  </si>
+  <si>
+    <t>0.4752223436</t>
+  </si>
+  <si>
+    <t>0.022322284</t>
+  </si>
+  <si>
+    <t>0.0076643035</t>
+  </si>
+  <si>
+    <t>0.3834067829</t>
+  </si>
+  <si>
+    <t>0.7842403611</t>
+  </si>
+  <si>
+    <t>0.4533371352</t>
+  </si>
+  <si>
+    <t>0.0319026633</t>
+  </si>
+  <si>
+    <t>0.0036405442</t>
+  </si>
+  <si>
+    <t>0.3127035831</t>
+  </si>
+  <si>
+    <t>0.721887472</t>
+  </si>
+  <si>
+    <t>0.4495049349</t>
+  </si>
+  <si>
+    <t>0.000958038</t>
+  </si>
+  <si>
+    <t>0.5260962449</t>
+  </si>
+  <si>
+    <t>0.4644065847</t>
+  </si>
+  <si>
+    <t>0.0005748228</t>
+  </si>
+  <si>
+    <t>0.2935428243</t>
+  </si>
+  <si>
+    <t>0.5019272767</t>
+  </si>
+  <si>
+    <t>0.4860498285</t>
+  </si>
+  <si>
+    <t>0.0295075685</t>
+  </si>
+  <si>
+    <t>0.003257329</t>
+  </si>
+  <si>
+    <t>0.2780226097</t>
+  </si>
+  <si>
+    <t>0.8206246848</t>
+  </si>
+  <si>
+    <t>0.392822447</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1446,6 +1933,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -1516,7 +2009,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1551,6 +2044,18 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1575,11 +2080,11 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="11" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1912,41 +2417,41 @@
     <col min="12" max="16384" width="51.33203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="20" customFormat="1" ht="66" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+    <row r="1" spans="1:12" s="12" customFormat="1" ht="66" x14ac:dyDescent="0.2">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="13" t="s">
         <v>284</v>
       </c>
-      <c r="D1" s="21" t="s">
+      <c r="D1" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="21" t="s">
+      <c r="E1" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="21" t="s">
+      <c r="F1" s="13" t="s">
         <v>385</v>
       </c>
-      <c r="G1" s="21" t="s">
+      <c r="G1" s="13" t="s">
         <v>386</v>
       </c>
-      <c r="H1" s="21" t="s">
+      <c r="H1" s="13" t="s">
         <v>387</v>
       </c>
-      <c r="I1" s="21" t="s">
+      <c r="I1" s="13" t="s">
         <v>388</v>
       </c>
-      <c r="J1" s="21" t="s">
-        <v>389</v>
-      </c>
-      <c r="K1" s="21" t="s">
+      <c r="J1" s="13" t="s">
+        <v>447</v>
+      </c>
+      <c r="K1" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="L1" s="21"/>
+      <c r="L1" s="13"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
@@ -1955,31 +2460,31 @@
       <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="22" t="s">
         <v>285</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="14" t="s">
         <v>350</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="14" t="s">
         <v>352</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="I2" s="14" t="s">
         <v>353</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" s="14" t="s">
         <v>354</v>
       </c>
-      <c r="K2" s="13" t="s">
+      <c r="K2" s="17" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1990,9 +2495,9 @@
       <c r="B3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="16"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
       <c r="F3" s="1" t="s">
         <v>346</v>
       </c>
@@ -2008,7 +2513,7 @@
       <c r="J3" s="1" t="s">
         <v>349</v>
       </c>
-      <c r="K3" s="14"/>
+      <c r="K3" s="18"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
@@ -2017,13 +2522,13 @@
       <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="16"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
       <c r="F4" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" s="14" t="s">
         <v>342</v>
       </c>
       <c r="H4" s="1" t="s">
@@ -2035,7 +2540,7 @@
       <c r="J4" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="K4" s="14"/>
+      <c r="K4" s="18"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
@@ -2044,22 +2549,22 @@
       <c r="B6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="C6" s="20" t="s">
         <v>286</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="D6" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="E6" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="14" t="s">
         <v>307</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="H6" s="14" t="s">
         <v>309</v>
       </c>
       <c r="I6" s="1" t="s">
@@ -2068,7 +2573,7 @@
       <c r="J6" s="1" t="s">
         <v>311</v>
       </c>
-      <c r="K6" s="14" t="s">
+      <c r="K6" s="18" t="s">
         <v>18</v>
       </c>
     </row>
@@ -2079,9 +2584,9 @@
       <c r="B7" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="16"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
+      <c r="C7" s="20"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
       <c r="F7" s="1" t="s">
         <v>302</v>
       </c>
@@ -2094,10 +2599,10 @@
       <c r="I7" s="1" t="s">
         <v>305</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="J7" s="14" t="s">
         <v>306</v>
       </c>
-      <c r="K7" s="14"/>
+      <c r="K7" s="18"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
@@ -2106,33 +2611,33 @@
       <c r="B8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="16"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
       <c r="F8" s="1" t="s">
         <v>297</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="G8" s="14" t="s">
         <v>298</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>299</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="I8" s="14" t="s">
         <v>300</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>301</v>
       </c>
-      <c r="K8" s="14"/>
+      <c r="K8" s="18"/>
     </row>
     <row r="10" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="17"/>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
       <c r="E10" s="11"/>
       <c r="F10" s="9"/>
       <c r="G10" s="9"/>
@@ -2148,16 +2653,31 @@
       <c r="B12" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="16" t="s">
+      <c r="C12" s="20" t="s">
         <v>287</v>
       </c>
-      <c r="D12" s="12" t="s">
+      <c r="D12" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="E12" s="12" t="s">
+      <c r="E12" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="K12" s="14" t="s">
+      <c r="F12" s="14" t="s">
+        <v>414</v>
+      </c>
+      <c r="G12" s="14" t="s">
+        <v>415</v>
+      </c>
+      <c r="H12" s="14" t="s">
+        <v>416</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="J12" s="14" t="s">
+        <v>418</v>
+      </c>
+      <c r="K12" s="18" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2168,10 +2688,25 @@
       <c r="B13" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="16"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="K13" s="14"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>411</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="K13" s="18"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
@@ -2180,10 +2715,25 @@
       <c r="B14" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="16"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="K14" s="14"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="I14" s="14" t="s">
+        <v>407</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="K14" s="18"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
@@ -2192,31 +2742,31 @@
       <c r="B16" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C16" s="16" t="s">
+      <c r="C16" s="20" t="s">
         <v>288</v>
       </c>
-      <c r="D16" s="12" t="s">
+      <c r="D16" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="E16" s="12" t="s">
+      <c r="E16" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="F16" s="14" t="s">
         <v>279</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="H16" s="1" t="s">
+      <c r="H16" s="14" t="s">
         <v>281</v>
       </c>
-      <c r="I16" s="1" t="s">
+      <c r="I16" s="14" t="s">
         <v>282</v>
       </c>
       <c r="J16" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="K16" s="14" t="s">
+      <c r="K16" s="18" t="s">
         <v>38</v>
       </c>
     </row>
@@ -2227,9 +2777,9 @@
       <c r="B17" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C17" s="16"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
       <c r="F17" s="1" t="s">
         <v>274</v>
       </c>
@@ -2242,10 +2792,10 @@
       <c r="I17" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="J17" s="1" t="s">
+      <c r="J17" s="14" t="s">
         <v>278</v>
       </c>
-      <c r="K17" s="14"/>
+      <c r="K17" s="18"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
@@ -2254,13 +2804,13 @@
       <c r="B18" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="16"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
       <c r="F18" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="G18" s="14" t="s">
         <v>270</v>
       </c>
       <c r="H18" s="1" t="s">
@@ -2272,7 +2822,7 @@
       <c r="J18" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="K18" s="14"/>
+      <c r="K18" s="18"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
@@ -2281,31 +2831,31 @@
       <c r="B20" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C20" s="16" t="s">
+      <c r="C20" s="20" t="s">
         <v>289</v>
       </c>
-      <c r="D20" s="12" t="s">
+      <c r="D20" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="E20" s="12" t="s">
+      <c r="E20" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="F20" s="1" t="s">
+      <c r="F20" s="14" t="s">
         <v>249</v>
       </c>
-      <c r="G20" s="1" t="s">
+      <c r="G20" s="14" t="s">
         <v>250</v>
       </c>
       <c r="H20" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="I20" s="1" t="s">
+      <c r="I20" s="14" t="s">
         <v>252</v>
       </c>
       <c r="J20" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="K20" s="14" t="s">
+      <c r="K20" s="18" t="s">
         <v>37</v>
       </c>
     </row>
@@ -2316,25 +2866,25 @@
       <c r="B21" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C21" s="16"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="12"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
       <c r="F21" s="1" t="s">
         <v>244</v>
       </c>
       <c r="G21" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="H21" s="1" t="s">
+      <c r="H21" s="14" t="s">
         <v>246</v>
       </c>
       <c r="I21" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="J21" s="1" t="s">
+      <c r="J21" s="15" t="s">
         <v>248</v>
       </c>
-      <c r="K21" s="14"/>
+      <c r="K21" s="18"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
@@ -2343,9 +2893,9 @@
       <c r="B22" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C22" s="16"/>
-      <c r="D22" s="12"/>
-      <c r="E22" s="12"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="16"/>
       <c r="F22" s="1" t="s">
         <v>239</v>
       </c>
@@ -2361,7 +2911,7 @@
       <c r="J22" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="K22" s="14"/>
+      <c r="K22" s="18"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
@@ -2370,28 +2920,28 @@
       <c r="B24" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C24" s="16" t="s">
+      <c r="C24" s="20" t="s">
         <v>290</v>
       </c>
-      <c r="D24" s="12" t="s">
+      <c r="D24" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="E24" s="12" t="s">
+      <c r="E24" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="F24" s="1" t="s">
+      <c r="F24" s="14" t="s">
         <v>365</v>
       </c>
-      <c r="G24" s="1" t="s">
+      <c r="G24" s="14" t="s">
         <v>366</v>
       </c>
-      <c r="H24" s="1" t="s">
+      <c r="H24" s="14" t="s">
         <v>367</v>
       </c>
-      <c r="I24" s="1" t="s">
+      <c r="I24" s="14" t="s">
         <v>368</v>
       </c>
-      <c r="J24" s="1" t="s">
+      <c r="J24" s="14" t="s">
         <v>369</v>
       </c>
     </row>
@@ -2402,9 +2952,9 @@
       <c r="B25" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C25" s="16"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="12"/>
+      <c r="C25" s="20"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="16"/>
       <c r="F25" s="1" t="s">
         <v>360</v>
       </c>
@@ -2428,9 +2978,9 @@
       <c r="B26" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C26" s="16"/>
-      <c r="D26" s="12"/>
-      <c r="E26" s="12"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="16"/>
       <c r="F26" s="1" t="s">
         <v>355</v>
       </c>
@@ -2454,19 +3004,19 @@
       <c r="B28" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C28" s="16" t="s">
+      <c r="C28" s="20" t="s">
         <v>291</v>
       </c>
-      <c r="D28" s="12" t="s">
+      <c r="D28" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="E28" s="12" t="s">
+      <c r="E28" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="F28" s="1" t="s">
+      <c r="F28" s="14" t="s">
         <v>336</v>
       </c>
-      <c r="G28" s="1" t="s">
+      <c r="G28" s="14" t="s">
         <v>337</v>
       </c>
       <c r="H28" s="1" t="s">
@@ -2475,7 +3025,7 @@
       <c r="I28" s="1" t="s">
         <v>339</v>
       </c>
-      <c r="J28" s="1" t="s">
+      <c r="J28" s="14" t="s">
         <v>340</v>
       </c>
     </row>
@@ -2486,9 +3036,9 @@
       <c r="B29" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C29" s="16"/>
-      <c r="D29" s="12"/>
-      <c r="E29" s="12"/>
+      <c r="C29" s="20"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
       <c r="F29" s="1" t="s">
         <v>331</v>
       </c>
@@ -2498,7 +3048,7 @@
       <c r="H29" s="1" t="s">
         <v>333</v>
       </c>
-      <c r="I29" s="1" t="s">
+      <c r="I29" s="14" t="s">
         <v>334</v>
       </c>
       <c r="J29" s="1" t="s">
@@ -2512,16 +3062,16 @@
       <c r="B30" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C30" s="16"/>
-      <c r="D30" s="12"/>
-      <c r="E30" s="12"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="16"/>
       <c r="F30" s="1" t="s">
         <v>326</v>
       </c>
       <c r="G30" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="H30" s="1" t="s">
+      <c r="H30" s="14" t="s">
         <v>328</v>
       </c>
       <c r="I30" s="1" t="s">
@@ -2538,14 +3088,29 @@
       <c r="B32" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C32" s="16" t="s">
+      <c r="C32" s="20" t="s">
         <v>292</v>
       </c>
-      <c r="D32" s="12" t="s">
+      <c r="D32" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="E32" s="12" t="s">
+      <c r="E32" s="16" t="s">
         <v>31</v>
+      </c>
+      <c r="F32" s="15" t="s">
+        <v>429</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="H32" s="14" t="s">
+        <v>431</v>
+      </c>
+      <c r="I32" s="15" t="s">
+        <v>432</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>433</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.2">
@@ -2555,9 +3120,24 @@
       <c r="B33" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C33" s="16"/>
-      <c r="D33" s="12"/>
-      <c r="E33" s="12"/>
+      <c r="C33" s="20"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="16"/>
+      <c r="F33" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="G33" s="14" t="s">
+        <v>425</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="I33" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="J33" s="14" t="s">
+        <v>428</v>
+      </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
@@ -2566,9 +3146,24 @@
       <c r="B34" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C34" s="16"/>
-      <c r="D34" s="12"/>
-      <c r="E34" s="12"/>
+      <c r="C34" s="20"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="16"/>
+      <c r="F34" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="H34" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="I34" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="J34" s="1" t="s">
+        <v>423</v>
+      </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
@@ -2577,29 +3172,29 @@
       <c r="B36" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C36" s="16" t="s">
+      <c r="C36" s="20" t="s">
         <v>293</v>
       </c>
-      <c r="D36" s="12" t="s">
+      <c r="D36" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="E36" s="12" t="s">
+      <c r="E36" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="F36" s="1" t="s">
+      <c r="F36" s="14" t="s">
+        <v>399</v>
+      </c>
+      <c r="G36" s="14" t="s">
         <v>400</v>
       </c>
-      <c r="G36" s="1" t="s">
+      <c r="H36" s="15" t="s">
         <v>401</v>
       </c>
-      <c r="H36" s="1" t="s">
+      <c r="I36" s="14" t="s">
         <v>402</v>
       </c>
-      <c r="I36" s="1" t="s">
+      <c r="J36" s="14" t="s">
         <v>403</v>
-      </c>
-      <c r="J36" s="1" t="s">
-        <v>404</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.2">
@@ -2609,23 +3204,23 @@
       <c r="B37" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C37" s="16"/>
-      <c r="D37" s="12"/>
-      <c r="E37" s="12"/>
+      <c r="C37" s="20"/>
+      <c r="D37" s="16"/>
+      <c r="E37" s="16"/>
       <c r="F37" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="G37" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="G37" s="1" t="s">
+      <c r="H37" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="H37" s="1" t="s">
+      <c r="I37" s="1" t="s">
         <v>397</v>
       </c>
-      <c r="I37" s="1" t="s">
+      <c r="J37" s="1" t="s">
         <v>398</v>
-      </c>
-      <c r="J37" s="1" t="s">
-        <v>399</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.2">
@@ -2635,32 +3230,32 @@
       <c r="B38" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C38" s="16"/>
-      <c r="D38" s="12"/>
-      <c r="E38" s="12"/>
+      <c r="C38" s="20"/>
+      <c r="D38" s="16"/>
+      <c r="E38" s="16"/>
       <c r="F38" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="G38" s="1" t="s">
         <v>390</v>
       </c>
-      <c r="G38" s="1" t="s">
+      <c r="H38" s="1" t="s">
         <v>391</v>
       </c>
-      <c r="H38" s="1" t="s">
+      <c r="I38" s="1" t="s">
         <v>392</v>
       </c>
-      <c r="I38" s="1" t="s">
+      <c r="J38" s="1" t="s">
         <v>393</v>
       </c>
-      <c r="J38" s="1" t="s">
-        <v>394</v>
-      </c>
     </row>
     <row r="40" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="17" t="s">
+      <c r="A40" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="B40" s="17"/>
-      <c r="C40" s="17"/>
-      <c r="D40" s="17"/>
+      <c r="B40" s="21"/>
+      <c r="C40" s="21"/>
+      <c r="D40" s="21"/>
       <c r="E40" s="11"/>
       <c r="F40" s="9"/>
       <c r="G40" s="9"/>
@@ -2676,31 +3271,31 @@
       <c r="B42" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C42" s="16" t="s">
+      <c r="C42" s="20" t="s">
         <v>294</v>
       </c>
-      <c r="D42" s="12" t="s">
+      <c r="D42" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="E42" s="12" t="s">
+      <c r="E42" s="16" t="s">
         <v>29</v>
       </c>
       <c r="F42" s="1" t="s">
         <v>321</v>
       </c>
-      <c r="G42" s="1" t="s">
+      <c r="G42" s="14" t="s">
         <v>322</v>
       </c>
-      <c r="H42" s="1" t="s">
+      <c r="H42" s="14" t="s">
         <v>323</v>
       </c>
-      <c r="I42" s="1" t="s">
+      <c r="I42" s="14" t="s">
         <v>324</v>
       </c>
       <c r="J42" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="K42" s="14" t="s">
+      <c r="K42" s="18" t="s">
         <v>32</v>
       </c>
     </row>
@@ -2711,10 +3306,10 @@
       <c r="B43" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C43" s="16"/>
-      <c r="D43" s="12"/>
-      <c r="E43" s="12"/>
-      <c r="F43" s="1" t="s">
+      <c r="C43" s="20"/>
+      <c r="D43" s="16"/>
+      <c r="E43" s="16"/>
+      <c r="F43" s="14" t="s">
         <v>317</v>
       </c>
       <c r="G43" s="1" t="s">
@@ -2726,10 +3321,10 @@
       <c r="I43" s="1" t="s">
         <v>319</v>
       </c>
-      <c r="J43" s="1" t="s">
+      <c r="J43" s="14" t="s">
         <v>320</v>
       </c>
-      <c r="K43" s="14"/>
+      <c r="K43" s="18"/>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
@@ -2738,9 +3333,9 @@
       <c r="B44" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C44" s="16"/>
-      <c r="D44" s="12"/>
-      <c r="E44" s="12"/>
+      <c r="C44" s="20"/>
+      <c r="D44" s="16"/>
+      <c r="E44" s="16"/>
       <c r="F44" s="1" t="s">
         <v>312</v>
       </c>
@@ -2756,7 +3351,7 @@
       <c r="J44" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="K44" s="14"/>
+      <c r="K44" s="18"/>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
@@ -2765,13 +3360,13 @@
       <c r="B46" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C46" s="16" t="s">
+      <c r="C46" s="20" t="s">
         <v>295</v>
       </c>
-      <c r="D46" s="12" t="s">
+      <c r="D46" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="E46" s="12" t="s">
+      <c r="E46" s="16" t="s">
         <v>30</v>
       </c>
       <c r="F46" s="1" t="s">
@@ -2783,13 +3378,13 @@
       <c r="H46" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="I46" s="1" t="s">
+      <c r="I46" s="14" t="s">
         <v>267</v>
       </c>
       <c r="J46" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="K46" s="14" t="s">
+      <c r="K46" s="18" t="s">
         <v>33</v>
       </c>
     </row>
@@ -2800,25 +3395,25 @@
       <c r="B47" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C47" s="16"/>
-      <c r="D47" s="12"/>
-      <c r="E47" s="12"/>
-      <c r="F47" s="1" t="s">
+      <c r="C47" s="20"/>
+      <c r="D47" s="16"/>
+      <c r="E47" s="16"/>
+      <c r="F47" s="14" t="s">
         <v>259</v>
       </c>
       <c r="G47" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="H47" s="1" t="s">
+      <c r="H47" s="14" t="s">
         <v>261</v>
       </c>
       <c r="I47" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="J47" s="1" t="s">
+      <c r="J47" s="14" t="s">
         <v>263</v>
       </c>
-      <c r="K47" s="14"/>
+      <c r="K47" s="18"/>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
@@ -2827,13 +3422,13 @@
       <c r="B48" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C48" s="16"/>
-      <c r="D48" s="12"/>
-      <c r="E48" s="12"/>
+      <c r="C48" s="20"/>
+      <c r="D48" s="16"/>
+      <c r="E48" s="16"/>
       <c r="F48" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="G48" s="1" t="s">
+      <c r="G48" s="14" t="s">
         <v>255</v>
       </c>
       <c r="H48" s="1" t="s">
@@ -2845,7 +3440,7 @@
       <c r="J48" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="K48" s="14"/>
+      <c r="K48" s="18"/>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
@@ -2854,25 +3449,25 @@
       <c r="B50" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C50" s="16" t="s">
+      <c r="C50" s="20" t="s">
         <v>296</v>
       </c>
-      <c r="D50" s="12" t="s">
+      <c r="D50" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="E50" s="12" t="s">
+      <c r="E50" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="F50" s="1" t="s">
+      <c r="F50" s="14" t="s">
         <v>380</v>
       </c>
       <c r="G50" s="1" t="s">
         <v>381</v>
       </c>
-      <c r="H50" s="1" t="s">
+      <c r="H50" s="14" t="s">
         <v>382</v>
       </c>
-      <c r="I50" s="1" t="s">
+      <c r="I50" s="14" t="s">
         <v>383</v>
       </c>
       <c r="J50" s="1" t="s">
@@ -2886,9 +3481,9 @@
       <c r="B51" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C51" s="16"/>
-      <c r="D51" s="12"/>
-      <c r="E51" s="12"/>
+      <c r="C51" s="20"/>
+      <c r="D51" s="16"/>
+      <c r="E51" s="16"/>
       <c r="F51" s="1" t="s">
         <v>375</v>
       </c>
@@ -2901,7 +3496,7 @@
       <c r="I51" s="1" t="s">
         <v>378</v>
       </c>
-      <c r="J51" s="1" t="s">
+      <c r="J51" s="14" t="s">
         <v>379</v>
       </c>
     </row>
@@ -2912,13 +3507,13 @@
       <c r="B52" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C52" s="16"/>
-      <c r="D52" s="12"/>
-      <c r="E52" s="12"/>
+      <c r="C52" s="20"/>
+      <c r="D52" s="16"/>
+      <c r="E52" s="16"/>
       <c r="F52" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="G52" s="1" t="s">
+      <c r="G52" s="15" t="s">
         <v>371</v>
       </c>
       <c r="H52" s="1" t="s">
@@ -2954,7 +3549,6 @@
     <mergeCell ref="A40:D40"/>
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="C2:C4"/>
-    <mergeCell ref="E12:E14"/>
     <mergeCell ref="E16:E18"/>
     <mergeCell ref="E20:E22"/>
     <mergeCell ref="C42:C44"/>
@@ -2978,6 +3572,7 @@
     <mergeCell ref="E42:E44"/>
     <mergeCell ref="E2:E4"/>
     <mergeCell ref="E6:E8"/>
+    <mergeCell ref="E12:E14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3002,41 +3597,41 @@
     <col min="12" max="16384" width="51.33203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="20" customFormat="1" ht="66" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+    <row r="1" spans="1:12" s="12" customFormat="1" ht="66" x14ac:dyDescent="0.2">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="13" t="s">
         <v>284</v>
       </c>
-      <c r="D1" s="21" t="s">
+      <c r="D1" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="21" t="s">
+      <c r="E1" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="21" t="s">
+      <c r="F1" s="13" t="s">
         <v>385</v>
       </c>
-      <c r="G1" s="21" t="s">
+      <c r="G1" s="13" t="s">
         <v>386</v>
       </c>
-      <c r="H1" s="21" t="s">
+      <c r="H1" s="13" t="s">
         <v>387</v>
       </c>
-      <c r="I1" s="21" t="s">
+      <c r="I1" s="13" t="s">
         <v>388</v>
       </c>
-      <c r="J1" s="21" t="s">
-        <v>389</v>
-      </c>
-      <c r="K1" s="21" t="s">
+      <c r="J1" s="13" t="s">
+        <v>446</v>
+      </c>
+      <c r="K1" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="L1" s="21"/>
+      <c r="L1" s="13"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
@@ -3045,16 +3640,31 @@
       <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="22" t="s">
         <v>285</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="K2" s="13" t="s">
+      <c r="F2" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>445</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="K2" s="17" t="s">
         <v>17</v>
       </c>
     </row>
@@ -3065,10 +3675,25 @@
       <c r="B3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="16"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="K3" s="14"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="K3" s="18"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
@@ -3077,10 +3702,25 @@
       <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="16"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="K4" s="14"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>435</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="K4" s="18"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
@@ -3089,16 +3729,31 @@
       <c r="B6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="C6" s="20" t="s">
         <v>286</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="D6" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="E6" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="K6" s="14" t="s">
+      <c r="F6" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>460</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>461</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="K6" s="18" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3109,10 +3764,25 @@
       <c r="B7" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="16"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="K7" s="14"/>
+      <c r="C7" s="20"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="K7" s="18"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
@@ -3121,18 +3791,33 @@
       <c r="B8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="16"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="K8" s="14"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>452</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="K8" s="18"/>
     </row>
     <row r="10" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="17"/>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
       <c r="E10" s="11"/>
       <c r="F10" s="9"/>
       <c r="G10" s="9"/>
@@ -3148,16 +3833,31 @@
       <c r="B12" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="16" t="s">
+      <c r="C12" s="20" t="s">
         <v>287</v>
       </c>
-      <c r="D12" s="12" t="s">
+      <c r="D12" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="E12" s="12" t="s">
+      <c r="E12" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="K12" s="14" t="s">
+      <c r="F12" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>475</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>477</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="K12" s="18" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3168,10 +3868,25 @@
       <c r="B13" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="16"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="K13" s="14"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>473</v>
+      </c>
+      <c r="K13" s="18"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
@@ -3180,10 +3895,25 @@
       <c r="B14" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="16"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="K14" s="14"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>465</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="K14" s="18"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
@@ -3192,16 +3922,31 @@
       <c r="B16" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C16" s="16" t="s">
+      <c r="C16" s="20" t="s">
         <v>288</v>
       </c>
-      <c r="D16" s="12" t="s">
+      <c r="D16" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="E16" s="12" t="s">
+      <c r="E16" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="K16" s="14" t="s">
+      <c r="F16" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>489</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>491</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="K16" s="18" t="s">
         <v>38</v>
       </c>
     </row>
@@ -3212,10 +3957,25 @@
       <c r="B17" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C17" s="16"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
-      <c r="K17" s="14"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="G17" s="24" t="s">
+        <v>484</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="K17" s="18"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
@@ -3224,10 +3984,25 @@
       <c r="B18" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="16"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="K18" s="14"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>481</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="K18" s="18"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
@@ -3236,16 +4011,16 @@
       <c r="B20" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C20" s="16" t="s">
+      <c r="C20" s="20" t="s">
         <v>289</v>
       </c>
-      <c r="D20" s="12" t="s">
+      <c r="D20" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="E20" s="12" t="s">
+      <c r="E20" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="K20" s="14" t="s">
+      <c r="K20" s="18" t="s">
         <v>37</v>
       </c>
     </row>
@@ -3256,10 +4031,10 @@
       <c r="B21" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C21" s="16"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="12"/>
-      <c r="K21" s="14"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
+      <c r="K21" s="18"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
@@ -3268,10 +4043,10 @@
       <c r="B22" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C22" s="16"/>
-      <c r="D22" s="12"/>
-      <c r="E22" s="12"/>
-      <c r="K22" s="14"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="16"/>
+      <c r="K22" s="18"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
@@ -3280,14 +4055,29 @@
       <c r="B24" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C24" s="16" t="s">
+      <c r="C24" s="20" t="s">
         <v>290</v>
       </c>
-      <c r="D24" s="12" t="s">
+      <c r="D24" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="E24" s="12" t="s">
+      <c r="E24" s="16" t="s">
         <v>34</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>500</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>501</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>503</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
@@ -3297,9 +4087,24 @@
       <c r="B25" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C25" s="16"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="12"/>
+      <c r="C25" s="20"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="1" t="s">
+        <v>495</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>497</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>499</v>
+      </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
@@ -3308,9 +4113,24 @@
       <c r="B26" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C26" s="16"/>
-      <c r="D26" s="12"/>
-      <c r="E26" s="12"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>493</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>494</v>
+      </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
@@ -3319,14 +4139,29 @@
       <c r="B28" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C28" s="16" t="s">
+      <c r="C28" s="20" t="s">
         <v>291</v>
       </c>
-      <c r="D28" s="12" t="s">
+      <c r="D28" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="E28" s="12" t="s">
+      <c r="E28" s="16" t="s">
         <v>35</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>512</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>513</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>514</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>515</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
@@ -3336,9 +4171,24 @@
       <c r="B29" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C29" s="16"/>
-      <c r="D29" s="12"/>
-      <c r="E29" s="12"/>
+      <c r="C29" s="20"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="1" t="s">
+        <v>507</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>508</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>509</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>510</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>511</v>
+      </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
@@ -3347,9 +4197,24 @@
       <c r="B30" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C30" s="16"/>
-      <c r="D30" s="12"/>
-      <c r="E30" s="12"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="H30" s="1" t="s">
+        <v>504</v>
+      </c>
+      <c r="I30" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="J30" s="1" t="s">
+        <v>506</v>
+      </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
@@ -3358,13 +4223,13 @@
       <c r="B32" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C32" s="16" t="s">
+      <c r="C32" s="20" t="s">
         <v>292</v>
       </c>
-      <c r="D32" s="12" t="s">
+      <c r="D32" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="E32" s="12" t="s">
+      <c r="E32" s="16" t="s">
         <v>31</v>
       </c>
     </row>
@@ -3375,9 +4240,9 @@
       <c r="B33" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C33" s="16"/>
-      <c r="D33" s="12"/>
-      <c r="E33" s="12"/>
+      <c r="C33" s="20"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="16"/>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
@@ -3386,9 +4251,9 @@
       <c r="B34" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C34" s="16"/>
-      <c r="D34" s="12"/>
-      <c r="E34" s="12"/>
+      <c r="C34" s="20"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="16"/>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
@@ -3397,14 +4262,29 @@
       <c r="B36" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C36" s="16" t="s">
+      <c r="C36" s="20" t="s">
         <v>293</v>
       </c>
-      <c r="D36" s="12" t="s">
+      <c r="D36" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="E36" s="12" t="s">
+      <c r="E36" s="16" t="s">
         <v>36</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>523</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>524</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>525</v>
+      </c>
+      <c r="J36" s="1" t="s">
+        <v>526</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.2">
@@ -3414,9 +4294,24 @@
       <c r="B37" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C37" s="16"/>
-      <c r="D37" s="12"/>
-      <c r="E37" s="12"/>
+      <c r="C37" s="20"/>
+      <c r="D37" s="16"/>
+      <c r="E37" s="16"/>
+      <c r="F37" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>519</v>
+      </c>
+      <c r="H37" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="I37" s="1" t="s">
+        <v>520</v>
+      </c>
+      <c r="J37" s="1" t="s">
+        <v>521</v>
+      </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
@@ -3425,17 +4320,32 @@
       <c r="B38" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C38" s="16"/>
-      <c r="D38" s="12"/>
-      <c r="E38" s="12"/>
+      <c r="C38" s="20"/>
+      <c r="D38" s="16"/>
+      <c r="E38" s="16"/>
+      <c r="F38" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="H38" s="1" t="s">
+        <v>516</v>
+      </c>
+      <c r="I38" s="1" t="s">
+        <v>517</v>
+      </c>
+      <c r="J38" s="1" t="s">
+        <v>518</v>
+      </c>
     </row>
     <row r="40" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="17" t="s">
+      <c r="A40" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="B40" s="17"/>
-      <c r="C40" s="17"/>
-      <c r="D40" s="17"/>
+      <c r="B40" s="21"/>
+      <c r="C40" s="21"/>
+      <c r="D40" s="21"/>
       <c r="E40" s="11"/>
       <c r="F40" s="9"/>
       <c r="G40" s="9"/>
@@ -3451,16 +4361,31 @@
       <c r="B42" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C42" s="16" t="s">
+      <c r="C42" s="20" t="s">
         <v>294</v>
       </c>
-      <c r="D42" s="12" t="s">
+      <c r="D42" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="E42" s="12" t="s">
+      <c r="E42" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="K42" s="14" t="s">
+      <c r="F42" s="1" t="s">
+        <v>536</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="H42" s="1" t="s">
+        <v>538</v>
+      </c>
+      <c r="I42" s="1" t="s">
+        <v>539</v>
+      </c>
+      <c r="J42" s="1" t="s">
+        <v>540</v>
+      </c>
+      <c r="K42" s="18" t="s">
         <v>32</v>
       </c>
     </row>
@@ -3471,10 +4396,25 @@
       <c r="B43" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C43" s="16"/>
-      <c r="D43" s="12"/>
-      <c r="E43" s="12"/>
-      <c r="K43" s="14"/>
+      <c r="C43" s="20"/>
+      <c r="D43" s="16"/>
+      <c r="E43" s="16"/>
+      <c r="F43" s="1" t="s">
+        <v>531</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>532</v>
+      </c>
+      <c r="H43" s="1" t="s">
+        <v>533</v>
+      </c>
+      <c r="I43" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="J43" s="1" t="s">
+        <v>535</v>
+      </c>
+      <c r="K43" s="18"/>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
@@ -3483,10 +4423,25 @@
       <c r="B44" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C44" s="16"/>
-      <c r="D44" s="12"/>
-      <c r="E44" s="12"/>
-      <c r="K44" s="14"/>
+      <c r="C44" s="20"/>
+      <c r="D44" s="16"/>
+      <c r="E44" s="16"/>
+      <c r="F44" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="H44" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="I44" s="1" t="s">
+        <v>529</v>
+      </c>
+      <c r="J44" s="1" t="s">
+        <v>530</v>
+      </c>
+      <c r="K44" s="18"/>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
@@ -3495,16 +4450,31 @@
       <c r="B46" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C46" s="16" t="s">
+      <c r="C46" s="20" t="s">
         <v>295</v>
       </c>
-      <c r="D46" s="12" t="s">
+      <c r="D46" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="E46" s="12" t="s">
+      <c r="E46" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="K46" s="14" t="s">
+      <c r="F46" s="1" t="s">
+        <v>550</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>551</v>
+      </c>
+      <c r="H46" s="1" t="s">
+        <v>552</v>
+      </c>
+      <c r="I46" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="J46" s="1" t="s">
+        <v>554</v>
+      </c>
+      <c r="K46" s="18" t="s">
         <v>33</v>
       </c>
     </row>
@@ -3515,10 +4485,25 @@
       <c r="B47" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C47" s="16"/>
-      <c r="D47" s="12"/>
-      <c r="E47" s="12"/>
-      <c r="K47" s="14"/>
+      <c r="C47" s="20"/>
+      <c r="D47" s="16"/>
+      <c r="E47" s="16"/>
+      <c r="F47" s="1" t="s">
+        <v>545</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>546</v>
+      </c>
+      <c r="H47" s="1" t="s">
+        <v>547</v>
+      </c>
+      <c r="I47" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="J47" s="1" t="s">
+        <v>549</v>
+      </c>
+      <c r="K47" s="18"/>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
@@ -3527,49 +4512,1199 @@
       <c r="B48" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C48" s="16"/>
-      <c r="D48" s="12"/>
-      <c r="E48" s="12"/>
-      <c r="K48" s="14"/>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="C48" s="20"/>
+      <c r="D48" s="16"/>
+      <c r="E48" s="16"/>
+      <c r="F48" s="1" t="s">
+        <v>541</v>
+      </c>
+      <c r="G48" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="H48" s="1" t="s">
+        <v>542</v>
+      </c>
+      <c r="I48" s="1" t="s">
+        <v>543</v>
+      </c>
+      <c r="J48" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="K48" s="18"/>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C50" s="16" t="s">
+      <c r="C50" s="20" t="s">
         <v>296</v>
       </c>
-      <c r="D50" s="12" t="s">
+      <c r="D50" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="E50" s="12" t="s">
+      <c r="E50" s="16" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F50" s="1" t="s">
+        <v>562</v>
+      </c>
+      <c r="G50" s="1" t="s">
+        <v>563</v>
+      </c>
+      <c r="H50" s="1" t="s">
+        <v>564</v>
+      </c>
+      <c r="I50" s="1" t="s">
+        <v>565</v>
+      </c>
+      <c r="J50" s="1" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C51" s="16"/>
-      <c r="D51" s="12"/>
-      <c r="E51" s="12"/>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="C51" s="20"/>
+      <c r="D51" s="16"/>
+      <c r="E51" s="16"/>
+      <c r="F51" s="1" t="s">
+        <v>558</v>
+      </c>
+      <c r="G51" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="H51" s="1" t="s">
+        <v>559</v>
+      </c>
+      <c r="I51" s="1" t="s">
+        <v>560</v>
+      </c>
+      <c r="J51" s="1" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C52" s="16"/>
-      <c r="D52" s="12"/>
-      <c r="E52" s="12"/>
+      <c r="C52" s="20"/>
+      <c r="D52" s="16"/>
+      <c r="E52" s="16"/>
+      <c r="F52" s="25" t="s">
+        <v>527</v>
+      </c>
+      <c r="G52" s="1" t="s">
+        <v>555</v>
+      </c>
+      <c r="H52" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="I52" s="1" t="s">
+        <v>556</v>
+      </c>
+      <c r="J52" s="1" t="s">
+        <v>557</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="45">
+    <mergeCell ref="K42:K44"/>
+    <mergeCell ref="C46:C48"/>
+    <mergeCell ref="D46:D48"/>
+    <mergeCell ref="E46:E48"/>
+    <mergeCell ref="K46:K48"/>
+    <mergeCell ref="C32:C34"/>
+    <mergeCell ref="D32:D34"/>
+    <mergeCell ref="E32:E34"/>
+    <mergeCell ref="C50:C52"/>
+    <mergeCell ref="D50:D52"/>
+    <mergeCell ref="E50:E52"/>
+    <mergeCell ref="C36:C38"/>
+    <mergeCell ref="D36:D38"/>
+    <mergeCell ref="E36:E38"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="C42:C44"/>
+    <mergeCell ref="D42:D44"/>
+    <mergeCell ref="E42:E44"/>
+    <mergeCell ref="C24:C26"/>
+    <mergeCell ref="D24:D26"/>
+    <mergeCell ref="E24:E26"/>
+    <mergeCell ref="C28:C30"/>
+    <mergeCell ref="D28:D30"/>
+    <mergeCell ref="E28:E30"/>
+    <mergeCell ref="K12:K14"/>
+    <mergeCell ref="C20:C22"/>
+    <mergeCell ref="D20:D22"/>
+    <mergeCell ref="E20:E22"/>
+    <mergeCell ref="K20:K22"/>
+    <mergeCell ref="C16:C18"/>
+    <mergeCell ref="D16:D18"/>
+    <mergeCell ref="E16:E18"/>
+    <mergeCell ref="K16:K18"/>
+    <mergeCell ref="C2:C4"/>
+    <mergeCell ref="D2:D4"/>
+    <mergeCell ref="E2:E4"/>
+    <mergeCell ref="K2:K4"/>
+    <mergeCell ref="C6:C8"/>
+    <mergeCell ref="D6:D8"/>
+    <mergeCell ref="E6:E8"/>
+    <mergeCell ref="K6:K8"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="C12:C14"/>
+    <mergeCell ref="D12:D14"/>
+    <mergeCell ref="E12:E14"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34A06E9C-6A0D-1745-934A-9CD3EA122E2E}">
+  <dimension ref="A1:L52"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="51.33203125" defaultRowHeight="21" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="26.1640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="17.6640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="34.5" style="1" customWidth="1"/>
+    <col min="4" max="4" width="50.33203125" style="10" customWidth="1"/>
+    <col min="5" max="5" width="50" style="10" customWidth="1"/>
+    <col min="6" max="6" width="24" style="1" customWidth="1"/>
+    <col min="7" max="7" width="23.1640625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="27.5" style="1" customWidth="1"/>
+    <col min="9" max="9" width="27.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="31.33203125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="68.33203125" style="6" customWidth="1"/>
+    <col min="12" max="16384" width="51.33203125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" s="12" customFormat="1" ht="66" x14ac:dyDescent="0.2">
+      <c r="A1" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>284</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>385</v>
+      </c>
+      <c r="G1" s="13" t="s">
+        <v>386</v>
+      </c>
+      <c r="H1" s="13" t="s">
+        <v>387</v>
+      </c>
+      <c r="I1" s="13" t="s">
+        <v>388</v>
+      </c>
+      <c r="J1" s="13" t="s">
+        <v>446</v>
+      </c>
+      <c r="K1" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="L1" s="13"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="22" t="s">
+        <v>285</v>
+      </c>
+      <c r="D2" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>445</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="K2" s="17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="20"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="K3" s="18"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="20"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>435</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="K4" s="18"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="20" t="s">
+        <v>286</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>460</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>461</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="K6" s="18" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="20"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="K7" s="18"/>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="20"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>452</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="K8" s="18"/>
+    </row>
+    <row r="10" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="9"/>
+      <c r="J10" s="9"/>
+      <c r="K10" s="11"/>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="20" t="s">
+        <v>287</v>
+      </c>
+      <c r="D12" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E12" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>475</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>477</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="K12" s="18" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" s="20"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>473</v>
+      </c>
+      <c r="K13" s="18"/>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="20"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>465</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="K14" s="18"/>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" s="20" t="s">
+        <v>288</v>
+      </c>
+      <c r="D16" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="E16" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>489</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>491</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="K16" s="18" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" s="20"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="G17" s="24" t="s">
+        <v>484</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="K17" s="18"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" s="20"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>481</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="K18" s="18"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A20" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="20" t="s">
+        <v>289</v>
+      </c>
+      <c r="D20" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="E20" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="K20" s="18" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A21" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" s="20"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
+      <c r="K21" s="18"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A22" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" s="20"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="16"/>
+      <c r="K22" s="18"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A24" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24" s="20" t="s">
+        <v>290</v>
+      </c>
+      <c r="D24" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="E24" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>500</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>501</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A25" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C25" s="20"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="1" t="s">
+        <v>495</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>497</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A26" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C26" s="20"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>493</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A28" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C28" s="20" t="s">
+        <v>291</v>
+      </c>
+      <c r="D28" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="E28" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>512</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>513</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>514</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A29" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C29" s="20"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="1" t="s">
+        <v>507</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>508</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>509</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>510</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A30" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C30" s="20"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="H30" s="1" t="s">
+        <v>504</v>
+      </c>
+      <c r="I30" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="J30" s="1" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A32" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C32" s="20" t="s">
+        <v>292</v>
+      </c>
+      <c r="D32" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="E32" s="16" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A33" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C33" s="20"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="16"/>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A34" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C34" s="20"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="16"/>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A36" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C36" s="20" t="s">
+        <v>293</v>
+      </c>
+      <c r="D36" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="E36" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>523</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>524</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>525</v>
+      </c>
+      <c r="J36" s="1" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A37" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C37" s="20"/>
+      <c r="D37" s="16"/>
+      <c r="E37" s="16"/>
+      <c r="F37" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>519</v>
+      </c>
+      <c r="H37" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="I37" s="1" t="s">
+        <v>520</v>
+      </c>
+      <c r="J37" s="1" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A38" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C38" s="20"/>
+      <c r="D38" s="16"/>
+      <c r="E38" s="16"/>
+      <c r="F38" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="H38" s="1" t="s">
+        <v>516</v>
+      </c>
+      <c r="I38" s="1" t="s">
+        <v>517</v>
+      </c>
+      <c r="J38" s="1" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="B40" s="21"/>
+      <c r="C40" s="21"/>
+      <c r="D40" s="21"/>
+      <c r="E40" s="11"/>
+      <c r="F40" s="9"/>
+      <c r="G40" s="9"/>
+      <c r="H40" s="9"/>
+      <c r="I40" s="9"/>
+      <c r="J40" s="9"/>
+      <c r="K40" s="11"/>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A42" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C42" s="20" t="s">
+        <v>294</v>
+      </c>
+      <c r="D42" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="E42" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>536</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="H42" s="1" t="s">
+        <v>538</v>
+      </c>
+      <c r="I42" s="1" t="s">
+        <v>539</v>
+      </c>
+      <c r="J42" s="1" t="s">
+        <v>540</v>
+      </c>
+      <c r="K42" s="18" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A43" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C43" s="20"/>
+      <c r="D43" s="16"/>
+      <c r="E43" s="16"/>
+      <c r="F43" s="1" t="s">
+        <v>531</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>532</v>
+      </c>
+      <c r="H43" s="1" t="s">
+        <v>533</v>
+      </c>
+      <c r="I43" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="J43" s="1" t="s">
+        <v>535</v>
+      </c>
+      <c r="K43" s="18"/>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A44" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C44" s="20"/>
+      <c r="D44" s="16"/>
+      <c r="E44" s="16"/>
+      <c r="F44" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="H44" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="I44" s="1" t="s">
+        <v>529</v>
+      </c>
+      <c r="J44" s="1" t="s">
+        <v>530</v>
+      </c>
+      <c r="K44" s="18"/>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A46" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C46" s="20" t="s">
+        <v>295</v>
+      </c>
+      <c r="D46" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="E46" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>550</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>551</v>
+      </c>
+      <c r="H46" s="1" t="s">
+        <v>552</v>
+      </c>
+      <c r="I46" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="J46" s="1" t="s">
+        <v>554</v>
+      </c>
+      <c r="K46" s="18" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A47" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C47" s="20"/>
+      <c r="D47" s="16"/>
+      <c r="E47" s="16"/>
+      <c r="F47" s="1" t="s">
+        <v>545</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>546</v>
+      </c>
+      <c r="H47" s="1" t="s">
+        <v>547</v>
+      </c>
+      <c r="I47" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="J47" s="1" t="s">
+        <v>549</v>
+      </c>
+      <c r="K47" s="18"/>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A48" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C48" s="20"/>
+      <c r="D48" s="16"/>
+      <c r="E48" s="16"/>
+      <c r="F48" s="1" t="s">
+        <v>541</v>
+      </c>
+      <c r="G48" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="H48" s="1" t="s">
+        <v>542</v>
+      </c>
+      <c r="I48" s="1" t="s">
+        <v>543</v>
+      </c>
+      <c r="J48" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="K48" s="18"/>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A50" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C50" s="20" t="s">
+        <v>296</v>
+      </c>
+      <c r="D50" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="E50" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>562</v>
+      </c>
+      <c r="G50" s="1" t="s">
+        <v>563</v>
+      </c>
+      <c r="H50" s="1" t="s">
+        <v>564</v>
+      </c>
+      <c r="I50" s="1" t="s">
+        <v>565</v>
+      </c>
+      <c r="J50" s="1" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A51" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C51" s="20"/>
+      <c r="D51" s="16"/>
+      <c r="E51" s="16"/>
+      <c r="F51" s="1" t="s">
+        <v>558</v>
+      </c>
+      <c r="G51" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="H51" s="1" t="s">
+        <v>559</v>
+      </c>
+      <c r="I51" s="1" t="s">
+        <v>560</v>
+      </c>
+      <c r="J51" s="1" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A52" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C52" s="20"/>
+      <c r="D52" s="16"/>
+      <c r="E52" s="16"/>
+      <c r="F52" s="25" t="s">
+        <v>527</v>
+      </c>
+      <c r="G52" s="1" t="s">
+        <v>555</v>
+      </c>
+      <c r="H52" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="I52" s="1" t="s">
+        <v>556</v>
+      </c>
+      <c r="J52" s="1" t="s">
+        <v>557</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="45">
@@ -3623,7 +5758,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F1BB833-377A-D44F-92A0-3B5384834C0E}">
   <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="38.6640625" defaultRowHeight="21" x14ac:dyDescent="0.2"/>
@@ -3664,13 +5799,13 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="23" t="s">
         <v>58</v>
       </c>
       <c r="D2" s="1" t="s">
@@ -3693,9 +5828,9 @@
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A3" s="14"/>
-      <c r="B3" s="16"/>
-      <c r="C3" s="19"/>
+      <c r="A3" s="18"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="23"/>
       <c r="D3" s="1" t="s">
         <v>46</v>
       </c>
@@ -3716,9 +5851,9 @@
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A4" s="14"/>
-      <c r="B4" s="16"/>
-      <c r="C4" s="19"/>
+      <c r="A4" s="18"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="23"/>
       <c r="D4" s="1" t="s">
         <v>47</v>
       </c>
@@ -3739,13 +5874,13 @@
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="18" t="s">
         <v>186</v>
       </c>
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="23" t="s">
         <v>57</v>
       </c>
       <c r="D6" s="1" t="s">
@@ -3768,9 +5903,9 @@
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A7" s="14"/>
-      <c r="B7" s="16"/>
-      <c r="C7" s="19"/>
+      <c r="A7" s="18"/>
+      <c r="B7" s="20"/>
+      <c r="C7" s="23"/>
       <c r="D7" s="1" t="s">
         <v>46</v>
       </c>
@@ -3791,9 +5926,9 @@
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A8" s="14"/>
-      <c r="B8" s="16"/>
-      <c r="C8" s="19"/>
+      <c r="A8" s="18"/>
+      <c r="B8" s="20"/>
+      <c r="C8" s="23"/>
       <c r="D8" s="1" t="s">
         <v>47</v>
       </c>
@@ -3814,13 +5949,13 @@
       </c>
     </row>
     <row r="10" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="18" t="s">
         <v>185</v>
       </c>
-      <c r="B10" s="16" t="s">
+      <c r="B10" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="23" t="s">
         <v>56</v>
       </c>
       <c r="D10" s="1" t="s">
@@ -3843,9 +5978,9 @@
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A11" s="14"/>
-      <c r="B11" s="16"/>
-      <c r="C11" s="19"/>
+      <c r="A11" s="18"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="23"/>
       <c r="D11" s="1" t="s">
         <v>46</v>
       </c>
@@ -3866,9 +6001,9 @@
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A12" s="14"/>
-      <c r="B12" s="16"/>
-      <c r="C12" s="19"/>
+      <c r="A12" s="18"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="23"/>
       <c r="D12" s="1" t="s">
         <v>47</v>
       </c>
@@ -3886,13 +6021,13 @@
       </c>
     </row>
     <row r="14" spans="1:9" s="3" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="14" t="s">
+      <c r="A14" s="18" t="s">
         <v>184</v>
       </c>
-      <c r="B14" s="16" t="s">
+      <c r="B14" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="C14" s="19" t="s">
+      <c r="C14" s="23" t="s">
         <v>55</v>
       </c>
       <c r="D14" s="3" t="s">
@@ -3915,9 +6050,9 @@
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A15" s="14"/>
-      <c r="B15" s="16"/>
-      <c r="C15" s="19"/>
+      <c r="A15" s="18"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="23"/>
       <c r="D15" s="1" t="s">
         <v>46</v>
       </c>
@@ -3938,9 +6073,9 @@
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A16" s="14"/>
-      <c r="B16" s="16"/>
-      <c r="C16" s="19"/>
+      <c r="A16" s="18"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="23"/>
       <c r="D16" s="1" t="s">
         <v>47</v>
       </c>
@@ -3961,13 +6096,13 @@
       </c>
     </row>
     <row r="18" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="14" t="s">
+      <c r="A18" s="18" t="s">
         <v>183</v>
       </c>
-      <c r="B18" s="16" t="s">
+      <c r="B18" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="C18" s="19" t="s">
+      <c r="C18" s="23" t="s">
         <v>59</v>
       </c>
       <c r="D18" s="1" t="s">
@@ -3990,9 +6125,9 @@
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A19" s="14"/>
-      <c r="B19" s="16"/>
-      <c r="C19" s="19"/>
+      <c r="A19" s="18"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="23"/>
       <c r="D19" s="1" t="s">
         <v>46</v>
       </c>
@@ -4013,9 +6148,9 @@
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A20" s="14"/>
-      <c r="B20" s="16"/>
-      <c r="C20" s="19"/>
+      <c r="A20" s="18"/>
+      <c r="B20" s="20"/>
+      <c r="C20" s="23"/>
       <c r="D20" s="1" t="s">
         <v>47</v>
       </c>
@@ -4033,13 +6168,13 @@
       </c>
     </row>
     <row r="22" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="14" t="s">
+      <c r="A22" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="B22" s="16" t="s">
+      <c r="B22" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="C22" s="19" t="s">
+      <c r="C22" s="23" t="s">
         <v>60</v>
       </c>
       <c r="D22" s="1" t="s">
@@ -4062,9 +6197,9 @@
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A23" s="14"/>
-      <c r="B23" s="16"/>
-      <c r="C23" s="19"/>
+      <c r="A23" s="18"/>
+      <c r="B23" s="20"/>
+      <c r="C23" s="23"/>
       <c r="D23" s="1" t="s">
         <v>46</v>
       </c>
@@ -4085,9 +6220,9 @@
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A24" s="14"/>
-      <c r="B24" s="16"/>
-      <c r="C24" s="19"/>
+      <c r="A24" s="18"/>
+      <c r="B24" s="20"/>
+      <c r="C24" s="23"/>
       <c r="D24" s="1" t="s">
         <v>47</v>
       </c>
@@ -4108,13 +6243,13 @@
       </c>
     </row>
     <row r="26" spans="1:9" s="3" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="19" t="s">
+      <c r="A26" s="23" t="s">
         <v>192</v>
       </c>
-      <c r="B26" s="19" t="s">
+      <c r="B26" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="C26" s="19" t="s">
+      <c r="C26" s="23" t="s">
         <v>122</v>
       </c>
       <c r="D26" s="3" t="s">
@@ -4137,9 +6272,9 @@
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A27" s="19"/>
-      <c r="B27" s="19"/>
-      <c r="C27" s="19"/>
+      <c r="A27" s="23"/>
+      <c r="B27" s="23"/>
+      <c r="C27" s="23"/>
       <c r="D27" s="1" t="s">
         <v>46</v>
       </c>
@@ -4160,9 +6295,9 @@
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A28" s="19"/>
-      <c r="B28" s="19"/>
-      <c r="C28" s="19"/>
+      <c r="A28" s="23"/>
+      <c r="B28" s="23"/>
+      <c r="C28" s="23"/>
       <c r="D28" s="1" t="s">
         <v>47</v>
       </c>
@@ -4187,13 +6322,13 @@
       <c r="B29" s="7"/>
     </row>
     <row r="30" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="19" t="s">
+      <c r="A30" s="23" t="s">
         <v>193</v>
       </c>
-      <c r="B30" s="19" t="s">
+      <c r="B30" s="23" t="s">
         <v>190</v>
       </c>
-      <c r="C30" s="19" t="s">
+      <c r="C30" s="23" t="s">
         <v>122</v>
       </c>
       <c r="D30" s="1" t="s">
@@ -4216,9 +6351,9 @@
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A31" s="19"/>
-      <c r="B31" s="19"/>
-      <c r="C31" s="19"/>
+      <c r="A31" s="23"/>
+      <c r="B31" s="23"/>
+      <c r="C31" s="23"/>
       <c r="D31" s="1" t="s">
         <v>46</v>
       </c>
@@ -4239,9 +6374,9 @@
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A32" s="19"/>
-      <c r="B32" s="19"/>
-      <c r="C32" s="19"/>
+      <c r="A32" s="23"/>
+      <c r="B32" s="23"/>
+      <c r="C32" s="23"/>
       <c r="D32" s="1" t="s">
         <v>47</v>
       </c>
@@ -4262,13 +6397,13 @@
       </c>
     </row>
     <row r="34" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="14" t="s">
+      <c r="A34" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="B34" s="19" t="s">
+      <c r="B34" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="C34" s="19" t="s">
+      <c r="C34" s="23" t="s">
         <v>180</v>
       </c>
       <c r="D34" s="1" t="s">
@@ -4291,9 +6426,9 @@
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A35" s="14"/>
-      <c r="B35" s="19"/>
-      <c r="C35" s="19"/>
+      <c r="A35" s="18"/>
+      <c r="B35" s="23"/>
+      <c r="C35" s="23"/>
       <c r="D35" s="1" t="s">
         <v>46</v>
       </c>
@@ -4314,9 +6449,9 @@
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A36" s="14"/>
-      <c r="B36" s="19"/>
-      <c r="C36" s="19"/>
+      <c r="A36" s="18"/>
+      <c r="B36" s="23"/>
+      <c r="C36" s="23"/>
       <c r="D36" s="1" t="s">
         <v>47</v>
       </c>
@@ -4337,13 +6472,13 @@
       </c>
     </row>
     <row r="38" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="14" t="s">
+      <c r="A38" s="18" t="s">
         <v>182</v>
       </c>
-      <c r="B38" s="14" t="s">
+      <c r="B38" s="18" t="s">
         <v>177</v>
       </c>
-      <c r="C38" s="19" t="s">
+      <c r="C38" s="23" t="s">
         <v>55</v>
       </c>
       <c r="D38" s="1" t="s">
@@ -4351,29 +6486,29 @@
       </c>
     </row>
     <row r="39" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="14"/>
-      <c r="B39" s="14"/>
-      <c r="C39" s="19"/>
+      <c r="A39" s="18"/>
+      <c r="B39" s="18"/>
+      <c r="C39" s="23"/>
       <c r="D39" s="1" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="14"/>
-      <c r="B40" s="14"/>
-      <c r="C40" s="19"/>
+      <c r="A40" s="18"/>
+      <c r="B40" s="18"/>
+      <c r="C40" s="23"/>
       <c r="D40" s="1" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="42" spans="1:9" s="3" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="14" t="s">
+      <c r="A42" s="18" t="s">
         <v>188</v>
       </c>
-      <c r="B42" s="14" t="s">
+      <c r="B42" s="18" t="s">
         <v>189</v>
       </c>
-      <c r="C42" s="19" t="s">
+      <c r="C42" s="23" t="s">
         <v>60</v>
       </c>
       <c r="D42" s="3" t="s">
@@ -4396,9 +6531,9 @@
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A43" s="14"/>
-      <c r="B43" s="14"/>
-      <c r="C43" s="19"/>
+      <c r="A43" s="18"/>
+      <c r="B43" s="18"/>
+      <c r="C43" s="23"/>
       <c r="D43" s="1" t="s">
         <v>46</v>
       </c>
@@ -4419,9 +6554,9 @@
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A44" s="14"/>
-      <c r="B44" s="14"/>
-      <c r="C44" s="19"/>
+      <c r="A44" s="18"/>
+      <c r="B44" s="18"/>
+      <c r="C44" s="23"/>
       <c r="D44" s="1" t="s">
         <v>47</v>
       </c>
@@ -4442,13 +6577,13 @@
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A46" s="14" t="s">
+      <c r="A46" s="18" t="s">
         <v>191</v>
       </c>
-      <c r="B46" s="14" t="s">
+      <c r="B46" s="18" t="s">
         <v>194</v>
       </c>
-      <c r="C46" s="19" t="s">
+      <c r="C46" s="23" t="s">
         <v>209</v>
       </c>
       <c r="D46" s="1" t="s">
@@ -4471,9 +6606,9 @@
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A47" s="14"/>
-      <c r="B47" s="14"/>
-      <c r="C47" s="19"/>
+      <c r="A47" s="18"/>
+      <c r="B47" s="18"/>
+      <c r="C47" s="23"/>
       <c r="D47" s="1" t="s">
         <v>46</v>
       </c>
@@ -4494,9 +6629,9 @@
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A48" s="14"/>
-      <c r="B48" s="14"/>
-      <c r="C48" s="19"/>
+      <c r="A48" s="18"/>
+      <c r="B48" s="18"/>
+      <c r="C48" s="23"/>
       <c r="D48" s="1" t="s">
         <v>47</v>
       </c>

</xml_diff>

<commit_message>
+ results for pretrained benchmarking
</commit_message>
<xml_diff>
--- a/benchmarking/search_for_best_combination/results_basic.xlsx
+++ b/benchmarking/search_for_best_combination/results_basic.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/deborahdore/Documents/political-debates-graph-analysis/benchmarking/search_for_best_combination/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F92F4EE-1B42-7D4D-961A-0011771379A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B844ED1-B5BA-B24B-BDFD-1E9A5AEBC9B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" activeTab="2" xr2:uid="{E2EDC037-19C4-FE46-A599-BB595128A04F}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="51200" windowHeight="28800" activeTab="2" xr2:uid="{E2EDC037-19C4-FE46-A599-BB595128A04F}"/>
   </bookViews>
   <sheets>
     <sheet name="Results BASIC" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1138" uniqueCount="593">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1018" uniqueCount="619">
   <si>
     <t>MODEL'S TYPE</t>
   </si>
@@ -1899,82 +1899,160 @@
     <t>0.392822447</t>
   </si>
   <si>
-    <t>0.3532118888</t>
-  </si>
-  <si>
-    <t>0.5520313963</t>
-  </si>
-  <si>
-    <t>0.4477544779</t>
-  </si>
-  <si>
-    <t>0.0041227229</t>
-  </si>
-  <si>
-    <t>0.2565675935</t>
-  </si>
-  <si>
-    <t>0.5509203869</t>
-  </si>
-  <si>
-    <t>0.4742471747</t>
-  </si>
-  <si>
-    <t>0.0209971237</t>
-  </si>
-  <si>
-    <t>0.0023010547</t>
-  </si>
-  <si>
-    <t>0.3390220518</t>
-  </si>
-  <si>
-    <t>0.8012936808</t>
-  </si>
-  <si>
-    <t>0.4286266132</t>
-  </si>
-  <si>
     <t>0.0005752637</t>
   </si>
   <si>
-    <t>0.6839884947</t>
-  </si>
-  <si>
-    <t>0.5024597125</t>
-  </si>
-  <si>
-    <t>0.4818168789</t>
-  </si>
-  <si>
-    <t>0.0620325983</t>
-  </si>
-  <si>
-    <t>0.0099712368</t>
-  </si>
-  <si>
-    <t>0.221093001</t>
-  </si>
-  <si>
-    <t>0.8361363854</t>
-  </si>
-  <si>
-    <t>0.3803620451</t>
-  </si>
-  <si>
-    <t>0.0265580058</t>
-  </si>
-  <si>
-    <t>0.0792905081</t>
-  </si>
-  <si>
-    <t>0.8982784427</t>
-  </si>
-  <si>
-    <t>0.4274209012</t>
-  </si>
-  <si>
-    <t>0.3460864386</t>
+    <t>0.0220517737</t>
+  </si>
+  <si>
+    <t>0.2607861937</t>
+  </si>
+  <si>
+    <t>0.5385824907</t>
+  </si>
+  <si>
+    <t>0.4074792697</t>
+  </si>
+  <si>
+    <t>0.083029722</t>
+  </si>
+  <si>
+    <t>0.2186001918</t>
+  </si>
+  <si>
+    <t>0.4934296451</t>
+  </si>
+  <si>
+    <t>0.4387721039</t>
+  </si>
+  <si>
+    <t>0.0911792905</t>
+  </si>
+  <si>
+    <t>0.2174496644</t>
+  </si>
+  <si>
+    <t>0.6639219361</t>
+  </si>
+  <si>
+    <t>0.4464361979</t>
+  </si>
+  <si>
+    <t>0.037171872</t>
+  </si>
+  <si>
+    <t>0.3494922399</t>
+  </si>
+  <si>
+    <t>0.4993320499</t>
+  </si>
+  <si>
+    <t>0.4255859946</t>
+  </si>
+  <si>
+    <t>0.044165549</t>
+  </si>
+  <si>
+    <t>0.002299291</t>
+  </si>
+  <si>
+    <t>0.3031232037</t>
+  </si>
+  <si>
+    <t>0.5179041185</t>
+  </si>
+  <si>
+    <t>0.4984225494</t>
+  </si>
+  <si>
+    <t>0.0420578655</t>
+  </si>
+  <si>
+    <t>0.1324008431</t>
+  </si>
+  <si>
+    <t>0.5080369989</t>
+  </si>
+  <si>
+    <t>0.3896901907</t>
+  </si>
+  <si>
+    <t>0.0255033557</t>
+  </si>
+  <si>
+    <t>0.5082465565</t>
+  </si>
+  <si>
+    <t>0.4652703056</t>
+  </si>
+  <si>
+    <t>0.0048897411</t>
+  </si>
+  <si>
+    <t>0.000671141</t>
+  </si>
+  <si>
+    <t>0.2851390221</t>
+  </si>
+  <si>
+    <t>0.5020983002</t>
+  </si>
+  <si>
+    <t>0.4881992368</t>
+  </si>
+  <si>
+    <t>0.0657718121</t>
+  </si>
+  <si>
+    <t>0.4945349952</t>
+  </si>
+  <si>
+    <t>0.5594059158</t>
+  </si>
+  <si>
+    <t>0.5183008532</t>
+  </si>
+  <si>
+    <t>0.0016286645</t>
+  </si>
+  <si>
+    <t>0.7286836559</t>
+  </si>
+  <si>
+    <t>0.4909162253</t>
+  </si>
+  <si>
+    <t>0.4915265534</t>
+  </si>
+  <si>
+    <t>0.0293159609</t>
+  </si>
+  <si>
+    <t>0.0035447404</t>
+  </si>
+  <si>
+    <t>0.3314811267</t>
+  </si>
+  <si>
+    <t>0.6347145411</t>
+  </si>
+  <si>
+    <t>0.4622564189</t>
+  </si>
+  <si>
+    <t>0.0333397203</t>
+  </si>
+  <si>
+    <t>0.0033531328</t>
+  </si>
+  <si>
+    <t>0.3939452002</t>
+  </si>
+  <si>
+    <t>0.6628225181</t>
+  </si>
+  <si>
+    <t>0.475877356</t>
   </si>
 </sst>
 </file>
@@ -2019,7 +2097,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2047,12 +2125,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2093,7 +2165,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2146,8 +2218,20 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2155,35 +2239,26 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2559,13 +2634,13 @@
       <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="24" t="s">
+      <c r="C2" s="22" t="s">
         <v>285</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="19" t="s">
         <v>15</v>
       </c>
       <c r="F2" s="14" t="s">
@@ -2583,7 +2658,7 @@
       <c r="J2" s="14" t="s">
         <v>354</v>
       </c>
-      <c r="K2" s="19" t="s">
+      <c r="K2" s="23" t="s">
         <v>17</v>
       </c>
     </row>
@@ -2594,9 +2669,9 @@
       <c r="B3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="22"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
       <c r="F3" s="1" t="s">
         <v>346</v>
       </c>
@@ -2612,7 +2687,7 @@
       <c r="J3" s="1" t="s">
         <v>349</v>
       </c>
-      <c r="K3" s="20"/>
+      <c r="K3" s="24"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
@@ -2621,9 +2696,9 @@
       <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="22"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
       <c r="F4" s="1" t="s">
         <v>341</v>
       </c>
@@ -2639,7 +2714,7 @@
       <c r="J4" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="K4" s="20"/>
+      <c r="K4" s="24"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
@@ -2648,13 +2723,13 @@
       <c r="B6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="22" t="s">
+      <c r="C6" s="18" t="s">
         <v>286</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="18" t="s">
+      <c r="E6" s="20" t="s">
         <v>15</v>
       </c>
       <c r="F6" s="14" t="s">
@@ -2672,7 +2747,7 @@
       <c r="J6" s="1" t="s">
         <v>311</v>
       </c>
-      <c r="K6" s="20" t="s">
+      <c r="K6" s="24" t="s">
         <v>18</v>
       </c>
     </row>
@@ -2683,9 +2758,9 @@
       <c r="B7" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="22"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="18"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="20"/>
+      <c r="E7" s="20"/>
       <c r="F7" s="1" t="s">
         <v>302</v>
       </c>
@@ -2701,7 +2776,7 @@
       <c r="J7" s="14" t="s">
         <v>306</v>
       </c>
-      <c r="K7" s="20"/>
+      <c r="K7" s="24"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
@@ -2710,9 +2785,9 @@
       <c r="B8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="22"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
       <c r="F8" s="1" t="s">
         <v>297</v>
       </c>
@@ -2728,15 +2803,15 @@
       <c r="J8" s="1" t="s">
         <v>301</v>
       </c>
-      <c r="K8" s="20"/>
+      <c r="K8" s="24"/>
     </row>
     <row r="10" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="23" t="s">
+      <c r="A10" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="23"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="23"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
       <c r="E10" s="11"/>
       <c r="F10" s="9"/>
       <c r="G10" s="9"/>
@@ -2752,13 +2827,13 @@
       <c r="B12" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="22" t="s">
+      <c r="C12" s="18" t="s">
         <v>287</v>
       </c>
-      <c r="D12" s="18" t="s">
+      <c r="D12" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="E12" s="18" t="s">
+      <c r="E12" s="20" t="s">
         <v>19</v>
       </c>
       <c r="F12" s="14" t="s">
@@ -2776,7 +2851,7 @@
       <c r="J12" s="14" t="s">
         <v>418</v>
       </c>
-      <c r="K12" s="20" t="s">
+      <c r="K12" s="24" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2787,9 +2862,9 @@
       <c r="B13" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="22"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
       <c r="F13" s="1" t="s">
         <v>409</v>
       </c>
@@ -2805,7 +2880,7 @@
       <c r="J13" s="1" t="s">
         <v>413</v>
       </c>
-      <c r="K13" s="20"/>
+      <c r="K13" s="24"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
@@ -2814,9 +2889,9 @@
       <c r="B14" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
       <c r="F14" s="1" t="s">
         <v>404</v>
       </c>
@@ -2832,7 +2907,7 @@
       <c r="J14" s="1" t="s">
         <v>408</v>
       </c>
-      <c r="K14" s="20"/>
+      <c r="K14" s="24"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
@@ -2841,13 +2916,13 @@
       <c r="B16" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C16" s="22" t="s">
+      <c r="C16" s="18" t="s">
         <v>288</v>
       </c>
-      <c r="D16" s="18" t="s">
+      <c r="D16" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="E16" s="18" t="s">
+      <c r="E16" s="20" t="s">
         <v>29</v>
       </c>
       <c r="F16" s="14" t="s">
@@ -2865,7 +2940,7 @@
       <c r="J16" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="K16" s="20" t="s">
+      <c r="K16" s="24" t="s">
         <v>38</v>
       </c>
     </row>
@@ -2876,9 +2951,9 @@
       <c r="B17" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C17" s="22"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20"/>
       <c r="F17" s="1" t="s">
         <v>274</v>
       </c>
@@ -2894,7 +2969,7 @@
       <c r="J17" s="14" t="s">
         <v>278</v>
       </c>
-      <c r="K17" s="20"/>
+      <c r="K17" s="24"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
@@ -2903,9 +2978,9 @@
       <c r="B18" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="22"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="20"/>
       <c r="F18" s="1" t="s">
         <v>269</v>
       </c>
@@ -2921,7 +2996,7 @@
       <c r="J18" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="K18" s="20"/>
+      <c r="K18" s="24"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
@@ -2930,13 +3005,13 @@
       <c r="B20" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C20" s="22" t="s">
+      <c r="C20" s="18" t="s">
         <v>289</v>
       </c>
-      <c r="D20" s="18" t="s">
+      <c r="D20" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="E20" s="18" t="s">
+      <c r="E20" s="20" t="s">
         <v>30</v>
       </c>
       <c r="F20" s="14" t="s">
@@ -2954,7 +3029,7 @@
       <c r="J20" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="K20" s="20" t="s">
+      <c r="K20" s="24" t="s">
         <v>37</v>
       </c>
     </row>
@@ -2965,9 +3040,9 @@
       <c r="B21" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C21" s="22"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="18"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
       <c r="F21" s="1" t="s">
         <v>244</v>
       </c>
@@ -2983,7 +3058,7 @@
       <c r="J21" s="15" t="s">
         <v>248</v>
       </c>
-      <c r="K21" s="20"/>
+      <c r="K21" s="24"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
@@ -2992,9 +3067,9 @@
       <c r="B22" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C22" s="22"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="18"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="20"/>
       <c r="F22" s="1" t="s">
         <v>239</v>
       </c>
@@ -3010,7 +3085,7 @@
       <c r="J22" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="K22" s="20"/>
+      <c r="K22" s="24"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
@@ -3019,13 +3094,13 @@
       <c r="B24" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C24" s="22" t="s">
+      <c r="C24" s="18" t="s">
         <v>290</v>
       </c>
-      <c r="D24" s="18" t="s">
+      <c r="D24" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="E24" s="18" t="s">
+      <c r="E24" s="20" t="s">
         <v>34</v>
       </c>
       <c r="F24" s="14" t="s">
@@ -3051,9 +3126,9 @@
       <c r="B25" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C25" s="22"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="18"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
       <c r="F25" s="1" t="s">
         <v>360</v>
       </c>
@@ -3077,9 +3152,9 @@
       <c r="B26" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C26" s="22"/>
-      <c r="D26" s="18"/>
-      <c r="E26" s="18"/>
+      <c r="C26" s="18"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
       <c r="F26" s="1" t="s">
         <v>355</v>
       </c>
@@ -3103,13 +3178,13 @@
       <c r="B28" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C28" s="22" t="s">
+      <c r="C28" s="18" t="s">
         <v>291</v>
       </c>
-      <c r="D28" s="18" t="s">
+      <c r="D28" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="E28" s="18" t="s">
+      <c r="E28" s="20" t="s">
         <v>35</v>
       </c>
       <c r="F28" s="14" t="s">
@@ -3135,9 +3210,9 @@
       <c r="B29" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C29" s="22"/>
-      <c r="D29" s="18"/>
-      <c r="E29" s="18"/>
+      <c r="C29" s="18"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="20"/>
       <c r="F29" s="1" t="s">
         <v>331</v>
       </c>
@@ -3161,9 +3236,9 @@
       <c r="B30" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C30" s="22"/>
-      <c r="D30" s="18"/>
-      <c r="E30" s="18"/>
+      <c r="C30" s="18"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="20"/>
       <c r="F30" s="1" t="s">
         <v>326</v>
       </c>
@@ -3187,13 +3262,13 @@
       <c r="B32" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C32" s="22" t="s">
+      <c r="C32" s="18" t="s">
         <v>292</v>
       </c>
-      <c r="D32" s="18" t="s">
+      <c r="D32" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="E32" s="18" t="s">
+      <c r="E32" s="20" t="s">
         <v>31</v>
       </c>
       <c r="F32" s="15" t="s">
@@ -3219,9 +3294,9 @@
       <c r="B33" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C33" s="22"/>
-      <c r="D33" s="18"/>
-      <c r="E33" s="18"/>
+      <c r="C33" s="18"/>
+      <c r="D33" s="20"/>
+      <c r="E33" s="20"/>
       <c r="F33" s="1" t="s">
         <v>424</v>
       </c>
@@ -3245,9 +3320,9 @@
       <c r="B34" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C34" s="22"/>
-      <c r="D34" s="18"/>
-      <c r="E34" s="18"/>
+      <c r="C34" s="18"/>
+      <c r="D34" s="20"/>
+      <c r="E34" s="20"/>
       <c r="F34" s="1" t="s">
         <v>419</v>
       </c>
@@ -3271,13 +3346,13 @@
       <c r="B36" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C36" s="22" t="s">
+      <c r="C36" s="18" t="s">
         <v>293</v>
       </c>
-      <c r="D36" s="18" t="s">
+      <c r="D36" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="E36" s="18" t="s">
+      <c r="E36" s="20" t="s">
         <v>36</v>
       </c>
       <c r="F36" s="14" t="s">
@@ -3303,9 +3378,9 @@
       <c r="B37" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C37" s="22"/>
-      <c r="D37" s="18"/>
-      <c r="E37" s="18"/>
+      <c r="C37" s="18"/>
+      <c r="D37" s="20"/>
+      <c r="E37" s="20"/>
       <c r="F37" s="1" t="s">
         <v>394</v>
       </c>
@@ -3329,9 +3404,9 @@
       <c r="B38" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C38" s="22"/>
-      <c r="D38" s="18"/>
-      <c r="E38" s="18"/>
+      <c r="C38" s="18"/>
+      <c r="D38" s="20"/>
+      <c r="E38" s="20"/>
       <c r="F38" s="1" t="s">
         <v>389</v>
       </c>
@@ -3349,12 +3424,12 @@
       </c>
     </row>
     <row r="40" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="23" t="s">
+      <c r="A40" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="B40" s="23"/>
-      <c r="C40" s="23"/>
-      <c r="D40" s="23"/>
+      <c r="B40" s="21"/>
+      <c r="C40" s="21"/>
+      <c r="D40" s="21"/>
       <c r="E40" s="11"/>
       <c r="F40" s="9"/>
       <c r="G40" s="9"/>
@@ -3370,13 +3445,13 @@
       <c r="B42" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C42" s="22" t="s">
+      <c r="C42" s="18" t="s">
         <v>294</v>
       </c>
-      <c r="D42" s="18" t="s">
+      <c r="D42" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="E42" s="18" t="s">
+      <c r="E42" s="20" t="s">
         <v>29</v>
       </c>
       <c r="F42" s="1" t="s">
@@ -3394,7 +3469,7 @@
       <c r="J42" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="K42" s="20" t="s">
+      <c r="K42" s="24" t="s">
         <v>32</v>
       </c>
     </row>
@@ -3405,9 +3480,9 @@
       <c r="B43" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C43" s="22"/>
-      <c r="D43" s="18"/>
-      <c r="E43" s="18"/>
+      <c r="C43" s="18"/>
+      <c r="D43" s="20"/>
+      <c r="E43" s="20"/>
       <c r="F43" s="14" t="s">
         <v>317</v>
       </c>
@@ -3423,7 +3498,7 @@
       <c r="J43" s="14" t="s">
         <v>320</v>
       </c>
-      <c r="K43" s="20"/>
+      <c r="K43" s="24"/>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
@@ -3432,9 +3507,9 @@
       <c r="B44" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C44" s="22"/>
-      <c r="D44" s="18"/>
-      <c r="E44" s="18"/>
+      <c r="C44" s="18"/>
+      <c r="D44" s="20"/>
+      <c r="E44" s="20"/>
       <c r="F44" s="1" t="s">
         <v>312</v>
       </c>
@@ -3450,7 +3525,7 @@
       <c r="J44" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="K44" s="20"/>
+      <c r="K44" s="24"/>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
@@ -3459,13 +3534,13 @@
       <c r="B46" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C46" s="22" t="s">
+      <c r="C46" s="18" t="s">
         <v>295</v>
       </c>
-      <c r="D46" s="18" t="s">
+      <c r="D46" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="E46" s="18" t="s">
+      <c r="E46" s="20" t="s">
         <v>30</v>
       </c>
       <c r="F46" s="1" t="s">
@@ -3483,7 +3558,7 @@
       <c r="J46" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="K46" s="20" t="s">
+      <c r="K46" s="24" t="s">
         <v>33</v>
       </c>
     </row>
@@ -3494,9 +3569,9 @@
       <c r="B47" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C47" s="22"/>
-      <c r="D47" s="18"/>
-      <c r="E47" s="18"/>
+      <c r="C47" s="18"/>
+      <c r="D47" s="20"/>
+      <c r="E47" s="20"/>
       <c r="F47" s="14" t="s">
         <v>259</v>
       </c>
@@ -3512,7 +3587,7 @@
       <c r="J47" s="14" t="s">
         <v>263</v>
       </c>
-      <c r="K47" s="20"/>
+      <c r="K47" s="24"/>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
@@ -3521,9 +3596,9 @@
       <c r="B48" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C48" s="22"/>
-      <c r="D48" s="18"/>
-      <c r="E48" s="18"/>
+      <c r="C48" s="18"/>
+      <c r="D48" s="20"/>
+      <c r="E48" s="20"/>
       <c r="F48" s="1" t="s">
         <v>254</v>
       </c>
@@ -3539,7 +3614,7 @@
       <c r="J48" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="K48" s="20"/>
+      <c r="K48" s="24"/>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
@@ -3548,13 +3623,13 @@
       <c r="B50" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C50" s="22" t="s">
+      <c r="C50" s="18" t="s">
         <v>296</v>
       </c>
-      <c r="D50" s="18" t="s">
+      <c r="D50" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="E50" s="18" t="s">
+      <c r="E50" s="20" t="s">
         <v>31</v>
       </c>
       <c r="F50" s="14" t="s">
@@ -3580,9 +3655,9 @@
       <c r="B51" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C51" s="22"/>
-      <c r="D51" s="18"/>
-      <c r="E51" s="18"/>
+      <c r="C51" s="18"/>
+      <c r="D51" s="20"/>
+      <c r="E51" s="20"/>
       <c r="F51" s="1" t="s">
         <v>375</v>
       </c>
@@ -3606,9 +3681,9 @@
       <c r="B52" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C52" s="22"/>
-      <c r="D52" s="18"/>
-      <c r="E52" s="18"/>
+      <c r="C52" s="18"/>
+      <c r="D52" s="20"/>
+      <c r="E52" s="20"/>
       <c r="F52" s="1" t="s">
         <v>370</v>
       </c>
@@ -3627,11 +3702,30 @@
     </row>
   </sheetData>
   <mergeCells count="45">
-    <mergeCell ref="C6:C8"/>
-    <mergeCell ref="C12:C14"/>
-    <mergeCell ref="C16:C18"/>
-    <mergeCell ref="C20:C22"/>
-    <mergeCell ref="C24:C26"/>
+    <mergeCell ref="E50:E52"/>
+    <mergeCell ref="K2:K4"/>
+    <mergeCell ref="K6:K8"/>
+    <mergeCell ref="K12:K14"/>
+    <mergeCell ref="K16:K18"/>
+    <mergeCell ref="K20:K22"/>
+    <mergeCell ref="K42:K44"/>
+    <mergeCell ref="K46:K48"/>
+    <mergeCell ref="E24:E26"/>
+    <mergeCell ref="E28:E30"/>
+    <mergeCell ref="E32:E34"/>
+    <mergeCell ref="E36:E38"/>
+    <mergeCell ref="E42:E44"/>
+    <mergeCell ref="E2:E4"/>
+    <mergeCell ref="E6:E8"/>
+    <mergeCell ref="E12:E14"/>
+    <mergeCell ref="E16:E18"/>
+    <mergeCell ref="E20:E22"/>
+    <mergeCell ref="C42:C44"/>
+    <mergeCell ref="C46:C48"/>
+    <mergeCell ref="C28:C30"/>
+    <mergeCell ref="C32:C34"/>
+    <mergeCell ref="C36:C38"/>
+    <mergeCell ref="E46:E48"/>
     <mergeCell ref="C50:C52"/>
     <mergeCell ref="D2:D4"/>
     <mergeCell ref="D6:D8"/>
@@ -3648,30 +3742,11 @@
     <mergeCell ref="A40:D40"/>
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="C2:C4"/>
-    <mergeCell ref="E16:E18"/>
-    <mergeCell ref="E20:E22"/>
-    <mergeCell ref="C42:C44"/>
-    <mergeCell ref="C46:C48"/>
-    <mergeCell ref="C28:C30"/>
-    <mergeCell ref="C32:C34"/>
-    <mergeCell ref="C36:C38"/>
-    <mergeCell ref="E46:E48"/>
-    <mergeCell ref="E50:E52"/>
-    <mergeCell ref="K2:K4"/>
-    <mergeCell ref="K6:K8"/>
-    <mergeCell ref="K12:K14"/>
-    <mergeCell ref="K16:K18"/>
-    <mergeCell ref="K20:K22"/>
-    <mergeCell ref="K42:K44"/>
-    <mergeCell ref="K46:K48"/>
-    <mergeCell ref="E24:E26"/>
-    <mergeCell ref="E28:E30"/>
-    <mergeCell ref="E32:E34"/>
-    <mergeCell ref="E36:E38"/>
-    <mergeCell ref="E42:E44"/>
-    <mergeCell ref="E2:E4"/>
-    <mergeCell ref="E6:E8"/>
-    <mergeCell ref="E12:E14"/>
+    <mergeCell ref="C6:C8"/>
+    <mergeCell ref="C12:C14"/>
+    <mergeCell ref="C16:C18"/>
+    <mergeCell ref="C20:C22"/>
+    <mergeCell ref="C24:C26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3739,13 +3814,13 @@
       <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="24" t="s">
+      <c r="C2" s="22" t="s">
         <v>285</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="19" t="s">
         <v>15</v>
       </c>
       <c r="F2" s="1" t="s">
@@ -3763,7 +3838,7 @@
       <c r="J2" s="1" t="s">
         <v>448</v>
       </c>
-      <c r="K2" s="19" t="s">
+      <c r="K2" s="23" t="s">
         <v>17</v>
       </c>
     </row>
@@ -3774,9 +3849,9 @@
       <c r="B3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="22"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
       <c r="F3" s="1" t="s">
         <v>438</v>
       </c>
@@ -3792,7 +3867,7 @@
       <c r="J3" s="1" t="s">
         <v>442</v>
       </c>
-      <c r="K3" s="20"/>
+      <c r="K3" s="24"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
@@ -3801,9 +3876,9 @@
       <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="22"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
       <c r="F4" s="1" t="s">
         <v>434</v>
       </c>
@@ -3819,7 +3894,7 @@
       <c r="J4" s="1" t="s">
         <v>437</v>
       </c>
-      <c r="K4" s="20"/>
+      <c r="K4" s="24"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
@@ -3828,13 +3903,13 @@
       <c r="B6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="22" t="s">
+      <c r="C6" s="18" t="s">
         <v>286</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="18" t="s">
+      <c r="E6" s="20" t="s">
         <v>15</v>
       </c>
       <c r="F6" s="1" t="s">
@@ -3852,7 +3927,7 @@
       <c r="J6" s="1" t="s">
         <v>463</v>
       </c>
-      <c r="K6" s="20" t="s">
+      <c r="K6" s="24" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3863,9 +3938,9 @@
       <c r="B7" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="22"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="18"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="20"/>
+      <c r="E7" s="20"/>
       <c r="F7" s="1" t="s">
         <v>454</v>
       </c>
@@ -3881,7 +3956,7 @@
       <c r="J7" s="1" t="s">
         <v>458</v>
       </c>
-      <c r="K7" s="20"/>
+      <c r="K7" s="24"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
@@ -3890,9 +3965,9 @@
       <c r="B8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="22"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
       <c r="F8" s="1" t="s">
         <v>449</v>
       </c>
@@ -3908,15 +3983,15 @@
       <c r="J8" s="1" t="s">
         <v>453</v>
       </c>
-      <c r="K8" s="20"/>
+      <c r="K8" s="24"/>
     </row>
     <row r="10" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="23" t="s">
+      <c r="A10" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="23"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="23"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
       <c r="E10" s="11"/>
       <c r="F10" s="9"/>
       <c r="G10" s="9"/>
@@ -3932,13 +4007,13 @@
       <c r="B12" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="22" t="s">
+      <c r="C12" s="18" t="s">
         <v>287</v>
       </c>
-      <c r="D12" s="18" t="s">
+      <c r="D12" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="E12" s="18" t="s">
+      <c r="E12" s="20" t="s">
         <v>19</v>
       </c>
       <c r="F12" s="1" t="s">
@@ -3956,7 +4031,7 @@
       <c r="J12" s="1" t="s">
         <v>478</v>
       </c>
-      <c r="K12" s="20" t="s">
+      <c r="K12" s="24" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3967,9 +4042,9 @@
       <c r="B13" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="22"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
       <c r="F13" s="1" t="s">
         <v>469</v>
       </c>
@@ -3985,7 +4060,7 @@
       <c r="J13" s="1" t="s">
         <v>473</v>
       </c>
-      <c r="K13" s="20"/>
+      <c r="K13" s="24"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
@@ -3994,9 +4069,9 @@
       <c r="B14" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
       <c r="F14" s="1" t="s">
         <v>464</v>
       </c>
@@ -4012,7 +4087,7 @@
       <c r="J14" s="1" t="s">
         <v>468</v>
       </c>
-      <c r="K14" s="20"/>
+      <c r="K14" s="24"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
@@ -4021,13 +4096,13 @@
       <c r="B16" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C16" s="22" t="s">
+      <c r="C16" s="18" t="s">
         <v>288</v>
       </c>
-      <c r="D16" s="18" t="s">
+      <c r="D16" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="E16" s="18" t="s">
+      <c r="E16" s="20" t="s">
         <v>29</v>
       </c>
       <c r="F16" s="1" t="s">
@@ -4045,7 +4120,7 @@
       <c r="J16" s="1" t="s">
         <v>492</v>
       </c>
-      <c r="K16" s="20" t="s">
+      <c r="K16" s="24" t="s">
         <v>38</v>
       </c>
     </row>
@@ -4056,9 +4131,9 @@
       <c r="B17" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C17" s="22"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20"/>
       <c r="F17" s="1" t="s">
         <v>483</v>
       </c>
@@ -4074,7 +4149,7 @@
       <c r="J17" s="1" t="s">
         <v>487</v>
       </c>
-      <c r="K17" s="20"/>
+      <c r="K17" s="24"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
@@ -4083,9 +4158,9 @@
       <c r="B18" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="22"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="20"/>
       <c r="F18" s="1" t="s">
         <v>479</v>
       </c>
@@ -4101,7 +4176,7 @@
       <c r="J18" s="1" t="s">
         <v>482</v>
       </c>
-      <c r="K18" s="20"/>
+      <c r="K18" s="24"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
@@ -4110,16 +4185,16 @@
       <c r="B20" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C20" s="22" t="s">
+      <c r="C20" s="18" t="s">
         <v>289</v>
       </c>
-      <c r="D20" s="18" t="s">
+      <c r="D20" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="E20" s="18" t="s">
+      <c r="E20" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="K20" s="20" t="s">
+      <c r="K20" s="24" t="s">
         <v>37</v>
       </c>
     </row>
@@ -4130,10 +4205,10 @@
       <c r="B21" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C21" s="22"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="18"/>
-      <c r="K21" s="20"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
+      <c r="K21" s="24"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
@@ -4142,10 +4217,10 @@
       <c r="B22" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C22" s="22"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="18"/>
-      <c r="K22" s="20"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="20"/>
+      <c r="K22" s="24"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
@@ -4154,13 +4229,13 @@
       <c r="B24" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C24" s="22" t="s">
+      <c r="C24" s="18" t="s">
         <v>290</v>
       </c>
-      <c r="D24" s="18" t="s">
+      <c r="D24" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="E24" s="18" t="s">
+      <c r="E24" s="20" t="s">
         <v>34</v>
       </c>
       <c r="F24" s="1" t="s">
@@ -4186,9 +4261,9 @@
       <c r="B25" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C25" s="22"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="18"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
       <c r="F25" s="1" t="s">
         <v>495</v>
       </c>
@@ -4212,9 +4287,9 @@
       <c r="B26" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C26" s="22"/>
-      <c r="D26" s="18"/>
-      <c r="E26" s="18"/>
+      <c r="C26" s="18"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
       <c r="F26" s="1" t="s">
         <v>464</v>
       </c>
@@ -4238,13 +4313,13 @@
       <c r="B28" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C28" s="22" t="s">
+      <c r="C28" s="18" t="s">
         <v>291</v>
       </c>
-      <c r="D28" s="18" t="s">
+      <c r="D28" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="E28" s="18" t="s">
+      <c r="E28" s="20" t="s">
         <v>35</v>
       </c>
       <c r="F28" s="1" t="s">
@@ -4270,9 +4345,9 @@
       <c r="B29" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C29" s="22"/>
-      <c r="D29" s="18"/>
-      <c r="E29" s="18"/>
+      <c r="C29" s="18"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="20"/>
       <c r="F29" s="1" t="s">
         <v>507</v>
       </c>
@@ -4296,9 +4371,9 @@
       <c r="B30" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C30" s="22"/>
-      <c r="D30" s="18"/>
-      <c r="E30" s="18"/>
+      <c r="C30" s="18"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="20"/>
       <c r="F30" s="1" t="s">
         <v>211</v>
       </c>
@@ -4322,13 +4397,13 @@
       <c r="B32" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C32" s="22" t="s">
+      <c r="C32" s="18" t="s">
         <v>292</v>
       </c>
-      <c r="D32" s="18" t="s">
+      <c r="D32" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="E32" s="18" t="s">
+      <c r="E32" s="20" t="s">
         <v>31</v>
       </c>
     </row>
@@ -4339,9 +4414,9 @@
       <c r="B33" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C33" s="22"/>
-      <c r="D33" s="18"/>
-      <c r="E33" s="18"/>
+      <c r="C33" s="18"/>
+      <c r="D33" s="20"/>
+      <c r="E33" s="20"/>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
@@ -4350,9 +4425,9 @@
       <c r="B34" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C34" s="22"/>
-      <c r="D34" s="18"/>
-      <c r="E34" s="18"/>
+      <c r="C34" s="18"/>
+      <c r="D34" s="20"/>
+      <c r="E34" s="20"/>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
@@ -4361,13 +4436,13 @@
       <c r="B36" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C36" s="22" t="s">
+      <c r="C36" s="18" t="s">
         <v>293</v>
       </c>
-      <c r="D36" s="18" t="s">
+      <c r="D36" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="E36" s="18" t="s">
+      <c r="E36" s="20" t="s">
         <v>36</v>
       </c>
       <c r="F36" s="1" t="s">
@@ -4393,9 +4468,9 @@
       <c r="B37" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C37" s="22"/>
-      <c r="D37" s="18"/>
-      <c r="E37" s="18"/>
+      <c r="C37" s="18"/>
+      <c r="D37" s="20"/>
+      <c r="E37" s="20"/>
       <c r="F37" s="1" t="s">
         <v>496</v>
       </c>
@@ -4419,9 +4494,9 @@
       <c r="B38" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C38" s="22"/>
-      <c r="D38" s="18"/>
-      <c r="E38" s="18"/>
+      <c r="C38" s="18"/>
+      <c r="D38" s="20"/>
+      <c r="E38" s="20"/>
       <c r="F38" s="1" t="s">
         <v>141</v>
       </c>
@@ -4439,12 +4514,12 @@
       </c>
     </row>
     <row r="40" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="23" t="s">
+      <c r="A40" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="B40" s="23"/>
-      <c r="C40" s="23"/>
-      <c r="D40" s="23"/>
+      <c r="B40" s="21"/>
+      <c r="C40" s="21"/>
+      <c r="D40" s="21"/>
       <c r="E40" s="11"/>
       <c r="F40" s="9"/>
       <c r="G40" s="9"/>
@@ -4460,13 +4535,13 @@
       <c r="B42" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C42" s="22" t="s">
+      <c r="C42" s="18" t="s">
         <v>294</v>
       </c>
-      <c r="D42" s="18" t="s">
+      <c r="D42" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="E42" s="18" t="s">
+      <c r="E42" s="20" t="s">
         <v>29</v>
       </c>
       <c r="F42" s="1" t="s">
@@ -4484,7 +4559,7 @@
       <c r="J42" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="K42" s="20" t="s">
+      <c r="K42" s="24" t="s">
         <v>32</v>
       </c>
     </row>
@@ -4495,9 +4570,9 @@
       <c r="B43" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C43" s="22"/>
-      <c r="D43" s="18"/>
-      <c r="E43" s="18"/>
+      <c r="C43" s="18"/>
+      <c r="D43" s="20"/>
+      <c r="E43" s="20"/>
       <c r="F43" s="1" t="s">
         <v>531</v>
       </c>
@@ -4513,7 +4588,7 @@
       <c r="J43" s="1" t="s">
         <v>535</v>
       </c>
-      <c r="K43" s="20"/>
+      <c r="K43" s="24"/>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
@@ -4522,9 +4597,9 @@
       <c r="B44" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C44" s="22"/>
-      <c r="D44" s="18"/>
-      <c r="E44" s="18"/>
+      <c r="C44" s="18"/>
+      <c r="D44" s="20"/>
+      <c r="E44" s="20"/>
       <c r="F44" s="1" t="s">
         <v>527</v>
       </c>
@@ -4540,7 +4615,7 @@
       <c r="J44" s="1" t="s">
         <v>530</v>
       </c>
-      <c r="K44" s="20"/>
+      <c r="K44" s="24"/>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
@@ -4549,13 +4624,13 @@
       <c r="B46" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C46" s="22" t="s">
+      <c r="C46" s="18" t="s">
         <v>295</v>
       </c>
-      <c r="D46" s="18" t="s">
+      <c r="D46" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="E46" s="18" t="s">
+      <c r="E46" s="20" t="s">
         <v>30</v>
       </c>
       <c r="F46" s="1" t="s">
@@ -4573,7 +4648,7 @@
       <c r="J46" s="1" t="s">
         <v>554</v>
       </c>
-      <c r="K46" s="20" t="s">
+      <c r="K46" s="24" t="s">
         <v>33</v>
       </c>
     </row>
@@ -4584,9 +4659,9 @@
       <c r="B47" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C47" s="22"/>
-      <c r="D47" s="18"/>
-      <c r="E47" s="18"/>
+      <c r="C47" s="18"/>
+      <c r="D47" s="20"/>
+      <c r="E47" s="20"/>
       <c r="F47" s="1" t="s">
         <v>545</v>
       </c>
@@ -4602,7 +4677,7 @@
       <c r="J47" s="1" t="s">
         <v>549</v>
       </c>
-      <c r="K47" s="20"/>
+      <c r="K47" s="24"/>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
@@ -4611,9 +4686,9 @@
       <c r="B48" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C48" s="22"/>
-      <c r="D48" s="18"/>
-      <c r="E48" s="18"/>
+      <c r="C48" s="18"/>
+      <c r="D48" s="20"/>
+      <c r="E48" s="20"/>
       <c r="F48" s="1" t="s">
         <v>541</v>
       </c>
@@ -4629,7 +4704,7 @@
       <c r="J48" s="1" t="s">
         <v>544</v>
       </c>
-      <c r="K48" s="20"/>
+      <c r="K48" s="24"/>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
@@ -4638,13 +4713,13 @@
       <c r="B50" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C50" s="22" t="s">
+      <c r="C50" s="18" t="s">
         <v>296</v>
       </c>
-      <c r="D50" s="18" t="s">
+      <c r="D50" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="E50" s="18" t="s">
+      <c r="E50" s="20" t="s">
         <v>31</v>
       </c>
       <c r="F50" s="1" t="s">
@@ -4670,9 +4745,9 @@
       <c r="B51" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C51" s="22"/>
-      <c r="D51" s="18"/>
-      <c r="E51" s="18"/>
+      <c r="C51" s="18"/>
+      <c r="D51" s="20"/>
+      <c r="E51" s="20"/>
       <c r="F51" s="1" t="s">
         <v>558</v>
       </c>
@@ -4696,9 +4771,9 @@
       <c r="B52" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C52" s="22"/>
-      <c r="D52" s="18"/>
-      <c r="E52" s="18"/>
+      <c r="C52" s="18"/>
+      <c r="D52" s="20"/>
+      <c r="E52" s="20"/>
       <c r="F52" s="17" t="s">
         <v>527</v>
       </c>
@@ -4717,11 +4792,33 @@
     </row>
   </sheetData>
   <mergeCells count="45">
-    <mergeCell ref="K42:K44"/>
-    <mergeCell ref="C46:C48"/>
-    <mergeCell ref="D46:D48"/>
-    <mergeCell ref="E46:E48"/>
-    <mergeCell ref="K46:K48"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="C12:C14"/>
+    <mergeCell ref="D12:D14"/>
+    <mergeCell ref="E12:E14"/>
+    <mergeCell ref="C2:C4"/>
+    <mergeCell ref="D2:D4"/>
+    <mergeCell ref="E2:E4"/>
+    <mergeCell ref="K2:K4"/>
+    <mergeCell ref="C6:C8"/>
+    <mergeCell ref="D6:D8"/>
+    <mergeCell ref="E6:E8"/>
+    <mergeCell ref="K6:K8"/>
+    <mergeCell ref="K12:K14"/>
+    <mergeCell ref="C20:C22"/>
+    <mergeCell ref="D20:D22"/>
+    <mergeCell ref="E20:E22"/>
+    <mergeCell ref="K20:K22"/>
+    <mergeCell ref="C16:C18"/>
+    <mergeCell ref="D16:D18"/>
+    <mergeCell ref="E16:E18"/>
+    <mergeCell ref="K16:K18"/>
+    <mergeCell ref="C24:C26"/>
+    <mergeCell ref="D24:D26"/>
+    <mergeCell ref="E24:E26"/>
+    <mergeCell ref="C28:C30"/>
+    <mergeCell ref="D28:D30"/>
+    <mergeCell ref="E28:E30"/>
     <mergeCell ref="C32:C34"/>
     <mergeCell ref="D32:D34"/>
     <mergeCell ref="E32:E34"/>
@@ -4735,33 +4832,11 @@
     <mergeCell ref="C42:C44"/>
     <mergeCell ref="D42:D44"/>
     <mergeCell ref="E42:E44"/>
-    <mergeCell ref="C24:C26"/>
-    <mergeCell ref="D24:D26"/>
-    <mergeCell ref="E24:E26"/>
-    <mergeCell ref="C28:C30"/>
-    <mergeCell ref="D28:D30"/>
-    <mergeCell ref="E28:E30"/>
-    <mergeCell ref="K12:K14"/>
-    <mergeCell ref="C20:C22"/>
-    <mergeCell ref="D20:D22"/>
-    <mergeCell ref="E20:E22"/>
-    <mergeCell ref="K20:K22"/>
-    <mergeCell ref="C16:C18"/>
-    <mergeCell ref="D16:D18"/>
-    <mergeCell ref="E16:E18"/>
-    <mergeCell ref="K16:K18"/>
-    <mergeCell ref="K2:K4"/>
-    <mergeCell ref="C6:C8"/>
-    <mergeCell ref="D6:D8"/>
-    <mergeCell ref="E6:E8"/>
-    <mergeCell ref="K6:K8"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="C12:C14"/>
-    <mergeCell ref="D12:D14"/>
-    <mergeCell ref="E12:E14"/>
-    <mergeCell ref="C2:C4"/>
-    <mergeCell ref="D2:D4"/>
-    <mergeCell ref="E2:E4"/>
+    <mergeCell ref="K42:K44"/>
+    <mergeCell ref="C46:C48"/>
+    <mergeCell ref="D46:D48"/>
+    <mergeCell ref="E46:E48"/>
+    <mergeCell ref="K46:K48"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4829,31 +4904,31 @@
       <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="24" t="s">
+      <c r="C2" s="22" t="s">
         <v>285</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="14" t="s">
-        <v>443</v>
+      <c r="F2" s="1" t="s">
+        <v>576</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>444</v>
+        <v>577</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>445</v>
+        <v>578</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>448</v>
-      </c>
-      <c r="K2" s="19" t="s">
+        <v>579</v>
+      </c>
+      <c r="K2" s="23" t="s">
         <v>17</v>
       </c>
     </row>
@@ -4864,25 +4939,25 @@
       <c r="B3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="22"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
       <c r="F3" s="1" t="s">
-        <v>438</v>
+        <v>572</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>439</v>
+        <v>567</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>440</v>
+        <v>573</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>441</v>
+        <v>574</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>442</v>
-      </c>
-      <c r="K3" s="20"/>
+        <v>575</v>
+      </c>
+      <c r="K3" s="24"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
@@ -4891,25 +4966,25 @@
       <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="22"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
       <c r="F4" s="1" t="s">
-        <v>434</v>
+        <v>568</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>108</v>
+        <v>211</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>435</v>
+        <v>569</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>436</v>
+        <v>570</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>437</v>
-      </c>
-      <c r="K4" s="20"/>
+        <v>571</v>
+      </c>
+      <c r="K4" s="24"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
@@ -4918,31 +4993,31 @@
       <c r="B6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="22" t="s">
+      <c r="C6" s="18" t="s">
         <v>286</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="18" t="s">
+      <c r="E6" s="20" t="s">
         <v>15</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>459</v>
+        <v>589</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>460</v>
+        <v>555</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>461</v>
+        <v>590</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>462</v>
-      </c>
-      <c r="J6" s="14" t="s">
-        <v>463</v>
-      </c>
-      <c r="K6" s="20" t="s">
+        <v>591</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>592</v>
+      </c>
+      <c r="K6" s="24" t="s">
         <v>18</v>
       </c>
     </row>
@@ -4953,25 +5028,25 @@
       <c r="B7" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="22"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="18"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="20"/>
+      <c r="E7" s="20"/>
       <c r="F7" s="1" t="s">
-        <v>454</v>
+        <v>584</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>455</v>
+        <v>585</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>456</v>
+        <v>586</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>457</v>
+        <v>587</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>458</v>
-      </c>
-      <c r="K7" s="20"/>
+        <v>588</v>
+      </c>
+      <c r="K7" s="24"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
@@ -4980,33 +5055,33 @@
       <c r="B8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="22"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
       <c r="F8" s="1" t="s">
-        <v>449</v>
+        <v>580</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>450</v>
+        <v>211</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>451</v>
+        <v>581</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>452</v>
+        <v>582</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>453</v>
-      </c>
-      <c r="K8" s="20"/>
+        <v>583</v>
+      </c>
+      <c r="K8" s="24"/>
     </row>
     <row r="10" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="23" t="s">
+      <c r="A10" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="23"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="23"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
       <c r="E10" s="11"/>
       <c r="F10" s="9"/>
       <c r="G10" s="9"/>
@@ -5022,31 +5097,31 @@
       <c r="B12" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="22" t="s">
+      <c r="C12" s="18" t="s">
         <v>287</v>
       </c>
-      <c r="D12" s="18" t="s">
+      <c r="D12" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="E12" s="18" t="s">
+      <c r="E12" s="20" t="s">
         <v>19</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>474</v>
+        <v>601</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>475</v>
+        <v>439</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>476</v>
+        <v>602</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>477</v>
+        <v>603</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>478</v>
-      </c>
-      <c r="K12" s="20" t="s">
+        <v>604</v>
+      </c>
+      <c r="K12" s="24" t="s">
         <v>20</v>
       </c>
     </row>
@@ -5057,25 +5132,25 @@
       <c r="B13" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="22"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
       <c r="F13" s="1" t="s">
-        <v>469</v>
+        <v>596</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>470</v>
+        <v>597</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>471</v>
+        <v>598</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>472</v>
+        <v>599</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>473</v>
-      </c>
-      <c r="K13" s="20"/>
+        <v>600</v>
+      </c>
+      <c r="K13" s="24"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
@@ -5084,25 +5159,25 @@
       <c r="B14" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
       <c r="F14" s="1" t="s">
-        <v>464</v>
+        <v>141</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>465</v>
+        <v>74</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>466</v>
+        <v>593</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>467</v>
+        <v>594</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>468</v>
-      </c>
-      <c r="K14" s="20"/>
+        <v>595</v>
+      </c>
+      <c r="K14" s="24"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
@@ -5111,31 +5186,16 @@
       <c r="B16" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C16" s="22" t="s">
+      <c r="C16" s="18" t="s">
         <v>288</v>
       </c>
-      <c r="D16" s="18" t="s">
+      <c r="D16" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="E16" s="18" t="s">
+      <c r="E16" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="F16" s="1" t="s">
-        <v>488</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>489</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>490</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>491</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>492</v>
-      </c>
-      <c r="K16" s="20" t="s">
+      <c r="K16" s="24" t="s">
         <v>38</v>
       </c>
     </row>
@@ -5146,25 +5206,11 @@
       <c r="B17" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C17" s="22"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="1" t="s">
-        <v>483</v>
-      </c>
-      <c r="G17" s="16" t="s">
-        <v>484</v>
-      </c>
-      <c r="H17" s="1" t="s">
-        <v>485</v>
-      </c>
-      <c r="I17" s="1" t="s">
-        <v>486</v>
-      </c>
-      <c r="J17" s="1" t="s">
-        <v>487</v>
-      </c>
-      <c r="K17" s="20"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20"/>
+      <c r="G17" s="16"/>
+      <c r="K17" s="24"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
@@ -5173,25 +5219,10 @@
       <c r="B18" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="22"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="1" t="s">
-        <v>479</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>480</v>
-      </c>
-      <c r="I18" s="1" t="s">
-        <v>481</v>
-      </c>
-      <c r="J18" s="1" t="s">
-        <v>482</v>
-      </c>
-      <c r="K18" s="20"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="20"/>
+      <c r="K18" s="24"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
@@ -5200,31 +5231,16 @@
       <c r="B20" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C20" s="22" t="s">
+      <c r="C20" s="18" t="s">
         <v>289</v>
       </c>
-      <c r="D20" s="18" t="s">
+      <c r="D20" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="E20" s="18" t="s">
+      <c r="E20" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="F20" s="1" t="s">
-        <v>574</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>575</v>
-      </c>
-      <c r="H20" s="1" t="s">
-        <v>576</v>
-      </c>
-      <c r="I20" s="1" t="s">
-        <v>577</v>
-      </c>
-      <c r="J20" s="1" t="s">
-        <v>578</v>
-      </c>
-      <c r="K20" s="20" t="s">
+      <c r="K20" s="24" t="s">
         <v>37</v>
       </c>
     </row>
@@ -5235,25 +5251,10 @@
       <c r="B21" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C21" s="22"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="18"/>
-      <c r="F21" s="1" t="s">
-        <v>470</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>570</v>
-      </c>
-      <c r="H21" s="1" t="s">
-        <v>571</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>572</v>
-      </c>
-      <c r="J21" s="1" t="s">
-        <v>573</v>
-      </c>
-      <c r="K21" s="20"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
+      <c r="K21" s="24"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
@@ -5262,25 +5263,10 @@
       <c r="B22" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C22" s="22"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="18"/>
-      <c r="F22" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="H22" s="1" t="s">
-        <v>567</v>
-      </c>
-      <c r="I22" s="1" t="s">
-        <v>568</v>
-      </c>
-      <c r="J22" s="1" t="s">
-        <v>569</v>
-      </c>
-      <c r="K22" s="20"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="20"/>
+      <c r="K22" s="24"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
@@ -5289,29 +5275,14 @@
       <c r="B24" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C24" s="22" t="s">
+      <c r="C24" s="18" t="s">
         <v>290</v>
       </c>
-      <c r="D24" s="18" t="s">
+      <c r="D24" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="E24" s="18" t="s">
+      <c r="E24" s="20" t="s">
         <v>34</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>500</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="H24" s="1" t="s">
-        <v>501</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>502</v>
-      </c>
-      <c r="J24" s="1" t="s">
-        <v>503</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
@@ -5321,24 +5292,9 @@
       <c r="B25" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C25" s="22"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="18"/>
-      <c r="F25" s="1" t="s">
-        <v>495</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>496</v>
-      </c>
-      <c r="H25" s="1" t="s">
-        <v>497</v>
-      </c>
-      <c r="I25" s="1" t="s">
-        <v>498</v>
-      </c>
-      <c r="J25" s="1" t="s">
-        <v>499</v>
-      </c>
+      <c r="C25" s="18"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
@@ -5347,24 +5303,9 @@
       <c r="B26" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C26" s="22"/>
-      <c r="D26" s="18"/>
-      <c r="E26" s="18"/>
-      <c r="F26" s="1" t="s">
-        <v>464</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="H26" s="1" t="s">
-        <v>241</v>
-      </c>
-      <c r="I26" s="1" t="s">
-        <v>493</v>
-      </c>
-      <c r="J26" s="1" t="s">
-        <v>494</v>
-      </c>
+      <c r="C26" s="18"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
@@ -5373,29 +5314,14 @@
       <c r="B28" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C28" s="22" t="s">
+      <c r="C28" s="18" t="s">
         <v>291</v>
       </c>
-      <c r="D28" s="18" t="s">
+      <c r="D28" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="E28" s="18" t="s">
+      <c r="E28" s="20" t="s">
         <v>35</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>512</v>
-      </c>
-      <c r="G28" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="H28" s="1" t="s">
-        <v>513</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>514</v>
-      </c>
-      <c r="J28" s="1" t="s">
-        <v>515</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
@@ -5405,24 +5331,9 @@
       <c r="B29" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C29" s="22"/>
-      <c r="D29" s="18"/>
-      <c r="E29" s="18"/>
-      <c r="F29" s="1" t="s">
-        <v>507</v>
-      </c>
-      <c r="G29" s="1" t="s">
-        <v>508</v>
-      </c>
-      <c r="H29" s="1" t="s">
-        <v>509</v>
-      </c>
-      <c r="I29" s="1" t="s">
-        <v>510</v>
-      </c>
-      <c r="J29" s="1" t="s">
-        <v>511</v>
-      </c>
+      <c r="C29" s="18"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="20"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
@@ -5431,24 +5342,9 @@
       <c r="B30" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C30" s="22"/>
-      <c r="D30" s="18"/>
-      <c r="E30" s="18"/>
-      <c r="F30" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="G30" s="1" t="s">
-        <v>351</v>
-      </c>
-      <c r="H30" s="1" t="s">
-        <v>504</v>
-      </c>
-      <c r="I30" s="1" t="s">
-        <v>505</v>
-      </c>
-      <c r="J30" s="1" t="s">
-        <v>506</v>
-      </c>
+      <c r="C30" s="18"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="20"/>
     </row>
     <row r="32" spans="1:11" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A32" s="26" t="s">
@@ -5466,21 +5362,8 @@
       <c r="E32" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="F32" s="26" t="s">
-        <v>588</v>
-      </c>
-      <c r="G32" s="29" t="s">
-        <v>589</v>
-      </c>
-      <c r="H32" s="26" t="s">
-        <v>591</v>
-      </c>
-      <c r="I32" s="29" t="s">
-        <v>590</v>
-      </c>
-      <c r="J32" s="26" t="s">
-        <v>592</v>
-      </c>
+      <c r="G32" s="29"/>
+      <c r="I32" s="29"/>
       <c r="K32" s="30"/>
     </row>
     <row r="33" spans="1:11" s="26" customFormat="1" x14ac:dyDescent="0.2">
@@ -5493,21 +5376,6 @@
       <c r="C33" s="27"/>
       <c r="D33" s="28"/>
       <c r="E33" s="28"/>
-      <c r="F33" s="26" t="s">
-        <v>583</v>
-      </c>
-      <c r="G33" s="26" t="s">
-        <v>584</v>
-      </c>
-      <c r="H33" s="26" t="s">
-        <v>585</v>
-      </c>
-      <c r="I33" s="26" t="s">
-        <v>586</v>
-      </c>
-      <c r="J33" s="26" t="s">
-        <v>587</v>
-      </c>
       <c r="K33" s="30"/>
     </row>
     <row r="34" spans="1:11" s="26" customFormat="1" x14ac:dyDescent="0.2">
@@ -5520,21 +5388,7 @@
       <c r="C34" s="27"/>
       <c r="D34" s="28"/>
       <c r="E34" s="28"/>
-      <c r="F34" s="26" t="s">
-        <v>579</v>
-      </c>
-      <c r="G34" s="26" t="s">
-        <v>475</v>
-      </c>
-      <c r="H34" s="29" t="s">
-        <v>580</v>
-      </c>
-      <c r="I34" s="26" t="s">
-        <v>581</v>
-      </c>
-      <c r="J34" s="26" t="s">
-        <v>582</v>
-      </c>
+      <c r="H34" s="29"/>
       <c r="K34" s="30"/>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.2">
@@ -5544,29 +5398,14 @@
       <c r="B36" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C36" s="22" t="s">
+      <c r="C36" s="18" t="s">
         <v>293</v>
       </c>
-      <c r="D36" s="18" t="s">
+      <c r="D36" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="E36" s="18" t="s">
+      <c r="E36" s="20" t="s">
         <v>36</v>
-      </c>
-      <c r="F36" s="1" t="s">
-        <v>522</v>
-      </c>
-      <c r="G36" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="H36" s="1" t="s">
-        <v>524</v>
-      </c>
-      <c r="I36" s="1" t="s">
-        <v>525</v>
-      </c>
-      <c r="J36" s="1" t="s">
-        <v>526</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.2">
@@ -5576,24 +5415,9 @@
       <c r="B37" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C37" s="22"/>
-      <c r="D37" s="18"/>
-      <c r="E37" s="18"/>
-      <c r="F37" s="1" t="s">
-        <v>496</v>
-      </c>
-      <c r="G37" s="1" t="s">
-        <v>519</v>
-      </c>
-      <c r="H37" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="I37" s="1" t="s">
-        <v>520</v>
-      </c>
-      <c r="J37" s="1" t="s">
-        <v>521</v>
-      </c>
+      <c r="C37" s="18"/>
+      <c r="D37" s="20"/>
+      <c r="E37" s="20"/>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
@@ -5602,32 +5426,17 @@
       <c r="B38" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C38" s="22"/>
-      <c r="D38" s="18"/>
-      <c r="E38" s="18"/>
-      <c r="F38" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="G38" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="H38" s="1" t="s">
-        <v>516</v>
-      </c>
-      <c r="I38" s="1" t="s">
-        <v>517</v>
-      </c>
-      <c r="J38" s="1" t="s">
-        <v>518</v>
-      </c>
+      <c r="C38" s="18"/>
+      <c r="D38" s="20"/>
+      <c r="E38" s="20"/>
     </row>
     <row r="40" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="23" t="s">
+      <c r="A40" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="B40" s="23"/>
-      <c r="C40" s="23"/>
-      <c r="D40" s="23"/>
+      <c r="B40" s="21"/>
+      <c r="C40" s="21"/>
+      <c r="D40" s="21"/>
       <c r="E40" s="11"/>
       <c r="F40" s="9"/>
       <c r="G40" s="9"/>
@@ -5643,31 +5452,31 @@
       <c r="B42" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C42" s="22" t="s">
+      <c r="C42" s="18" t="s">
         <v>294</v>
       </c>
-      <c r="D42" s="18" t="s">
+      <c r="D42" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="E42" s="18" t="s">
+      <c r="E42" s="20" t="s">
         <v>29</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>536</v>
+        <v>614</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>537</v>
+        <v>615</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>538</v>
+        <v>616</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>539</v>
+        <v>617</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>540</v>
-      </c>
-      <c r="K42" s="20" t="s">
+        <v>618</v>
+      </c>
+      <c r="K42" s="24" t="s">
         <v>32</v>
       </c>
     </row>
@@ -5678,25 +5487,25 @@
       <c r="B43" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C43" s="22"/>
-      <c r="D43" s="18"/>
-      <c r="E43" s="18"/>
+      <c r="C43" s="18"/>
+      <c r="D43" s="20"/>
+      <c r="E43" s="20"/>
       <c r="F43" s="1" t="s">
-        <v>531</v>
+        <v>609</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>532</v>
+        <v>610</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>533</v>
+        <v>611</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>534</v>
+        <v>612</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>535</v>
-      </c>
-      <c r="K43" s="20"/>
+        <v>613</v>
+      </c>
+      <c r="K43" s="24"/>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
@@ -5705,25 +5514,25 @@
       <c r="B44" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C44" s="22"/>
-      <c r="D44" s="18"/>
-      <c r="E44" s="18"/>
-      <c r="F44" s="1" t="s">
+      <c r="C44" s="18"/>
+      <c r="D44" s="20"/>
+      <c r="E44" s="20"/>
+      <c r="F44" s="31" t="s">
         <v>527</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>528</v>
+        <v>605</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>241</v>
+        <v>606</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>529</v>
+        <v>607</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>530</v>
-      </c>
-      <c r="K44" s="20"/>
+        <v>608</v>
+      </c>
+      <c r="K44" s="24"/>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
@@ -5732,31 +5541,16 @@
       <c r="B46" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C46" s="22" t="s">
+      <c r="C46" s="18" t="s">
         <v>295</v>
       </c>
-      <c r="D46" s="18" t="s">
+      <c r="D46" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="E46" s="18" t="s">
+      <c r="E46" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="F46" s="1" t="s">
-        <v>550</v>
-      </c>
-      <c r="G46" s="1" t="s">
-        <v>551</v>
-      </c>
-      <c r="H46" s="1" t="s">
-        <v>552</v>
-      </c>
-      <c r="I46" s="1" t="s">
-        <v>553</v>
-      </c>
-      <c r="J46" s="1" t="s">
-        <v>554</v>
-      </c>
-      <c r="K46" s="20" t="s">
+      <c r="K46" s="24" t="s">
         <v>33</v>
       </c>
     </row>
@@ -5767,25 +5561,10 @@
       <c r="B47" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C47" s="22"/>
-      <c r="D47" s="18"/>
-      <c r="E47" s="18"/>
-      <c r="F47" s="1" t="s">
-        <v>545</v>
-      </c>
-      <c r="G47" s="1" t="s">
-        <v>546</v>
-      </c>
-      <c r="H47" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="I47" s="1" t="s">
-        <v>548</v>
-      </c>
-      <c r="J47" s="1" t="s">
-        <v>549</v>
-      </c>
-      <c r="K47" s="20"/>
+      <c r="C47" s="18"/>
+      <c r="D47" s="20"/>
+      <c r="E47" s="20"/>
+      <c r="K47" s="24"/>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
@@ -5794,117 +5573,80 @@
       <c r="B48" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C48" s="22"/>
-      <c r="D48" s="18"/>
-      <c r="E48" s="18"/>
-      <c r="F48" s="1" t="s">
-        <v>541</v>
-      </c>
-      <c r="G48" s="1" t="s">
-        <v>455</v>
-      </c>
-      <c r="H48" s="1" t="s">
-        <v>542</v>
-      </c>
-      <c r="I48" s="1" t="s">
-        <v>543</v>
-      </c>
-      <c r="J48" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="K48" s="20"/>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="C48" s="18"/>
+      <c r="D48" s="20"/>
+      <c r="E48" s="20"/>
+      <c r="K48" s="24"/>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C50" s="22" t="s">
+      <c r="C50" s="18" t="s">
         <v>296</v>
       </c>
-      <c r="D50" s="18" t="s">
+      <c r="D50" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="E50" s="18" t="s">
+      <c r="E50" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="F50" s="1" t="s">
-        <v>562</v>
-      </c>
-      <c r="G50" s="1" t="s">
-        <v>563</v>
-      </c>
-      <c r="H50" s="1" t="s">
-        <v>564</v>
-      </c>
-      <c r="I50" s="1" t="s">
-        <v>565</v>
-      </c>
-      <c r="J50" s="1" t="s">
-        <v>566</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C51" s="22"/>
-      <c r="D51" s="18"/>
-      <c r="E51" s="18"/>
-      <c r="F51" s="1" t="s">
-        <v>558</v>
-      </c>
-      <c r="G51" s="1" t="s">
-        <v>455</v>
-      </c>
-      <c r="H51" s="1" t="s">
-        <v>559</v>
-      </c>
-      <c r="I51" s="1" t="s">
-        <v>560</v>
-      </c>
-      <c r="J51" s="1" t="s">
-        <v>561</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="C51" s="18"/>
+      <c r="D51" s="20"/>
+      <c r="E51" s="20"/>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C52" s="22"/>
-      <c r="D52" s="18"/>
-      <c r="E52" s="18"/>
-      <c r="F52" s="17" t="s">
-        <v>527</v>
-      </c>
-      <c r="G52" s="1" t="s">
-        <v>555</v>
-      </c>
-      <c r="H52" s="1" t="s">
-        <v>241</v>
-      </c>
-      <c r="I52" s="1" t="s">
-        <v>556</v>
-      </c>
-      <c r="J52" s="1" t="s">
-        <v>557</v>
-      </c>
+      <c r="C52" s="18"/>
+      <c r="D52" s="20"/>
+      <c r="E52" s="20"/>
+      <c r="F52" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="45">
-    <mergeCell ref="K42:K44"/>
-    <mergeCell ref="C46:C48"/>
-    <mergeCell ref="D46:D48"/>
-    <mergeCell ref="E46:E48"/>
-    <mergeCell ref="K46:K48"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="C12:C14"/>
+    <mergeCell ref="D12:D14"/>
+    <mergeCell ref="E12:E14"/>
+    <mergeCell ref="C2:C4"/>
+    <mergeCell ref="D2:D4"/>
+    <mergeCell ref="E2:E4"/>
+    <mergeCell ref="K2:K4"/>
+    <mergeCell ref="C6:C8"/>
+    <mergeCell ref="D6:D8"/>
+    <mergeCell ref="E6:E8"/>
+    <mergeCell ref="K6:K8"/>
+    <mergeCell ref="K12:K14"/>
+    <mergeCell ref="C20:C22"/>
+    <mergeCell ref="D20:D22"/>
+    <mergeCell ref="E20:E22"/>
+    <mergeCell ref="K20:K22"/>
+    <mergeCell ref="C16:C18"/>
+    <mergeCell ref="D16:D18"/>
+    <mergeCell ref="E16:E18"/>
+    <mergeCell ref="K16:K18"/>
+    <mergeCell ref="C24:C26"/>
+    <mergeCell ref="D24:D26"/>
+    <mergeCell ref="E24:E26"/>
+    <mergeCell ref="C28:C30"/>
+    <mergeCell ref="D28:D30"/>
+    <mergeCell ref="E28:E30"/>
     <mergeCell ref="C32:C34"/>
     <mergeCell ref="D32:D34"/>
     <mergeCell ref="E32:E34"/>
@@ -5918,33 +5660,11 @@
     <mergeCell ref="C42:C44"/>
     <mergeCell ref="D42:D44"/>
     <mergeCell ref="E42:E44"/>
-    <mergeCell ref="C24:C26"/>
-    <mergeCell ref="D24:D26"/>
-    <mergeCell ref="E24:E26"/>
-    <mergeCell ref="C28:C30"/>
-    <mergeCell ref="D28:D30"/>
-    <mergeCell ref="E28:E30"/>
-    <mergeCell ref="K12:K14"/>
-    <mergeCell ref="C20:C22"/>
-    <mergeCell ref="D20:D22"/>
-    <mergeCell ref="E20:E22"/>
-    <mergeCell ref="K20:K22"/>
-    <mergeCell ref="C16:C18"/>
-    <mergeCell ref="D16:D18"/>
-    <mergeCell ref="E16:E18"/>
-    <mergeCell ref="K16:K18"/>
-    <mergeCell ref="C2:C4"/>
-    <mergeCell ref="D2:D4"/>
-    <mergeCell ref="E2:E4"/>
-    <mergeCell ref="K2:K4"/>
-    <mergeCell ref="C6:C8"/>
-    <mergeCell ref="D6:D8"/>
-    <mergeCell ref="E6:E8"/>
-    <mergeCell ref="K6:K8"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="C12:C14"/>
-    <mergeCell ref="D12:D14"/>
-    <mergeCell ref="E12:E14"/>
+    <mergeCell ref="K42:K44"/>
+    <mergeCell ref="C46:C48"/>
+    <mergeCell ref="D46:D48"/>
+    <mergeCell ref="E46:E48"/>
+    <mergeCell ref="K46:K48"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5991,10 +5711,10 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="24" t="s">
         <v>187</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="18" t="s">
         <v>48</v>
       </c>
       <c r="C2" s="25" t="s">
@@ -6020,8 +5740,8 @@
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A3" s="20"/>
-      <c r="B3" s="22"/>
+      <c r="A3" s="24"/>
+      <c r="B3" s="18"/>
       <c r="C3" s="25"/>
       <c r="D3" s="1" t="s">
         <v>46</v>
@@ -6043,8 +5763,8 @@
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A4" s="20"/>
-      <c r="B4" s="22"/>
+      <c r="A4" s="24"/>
+      <c r="B4" s="18"/>
       <c r="C4" s="25"/>
       <c r="D4" s="1" t="s">
         <v>47</v>
@@ -6066,10 +5786,10 @@
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="24" t="s">
         <v>186</v>
       </c>
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="18" t="s">
         <v>49</v>
       </c>
       <c r="C6" s="25" t="s">
@@ -6095,8 +5815,8 @@
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A7" s="20"/>
-      <c r="B7" s="22"/>
+      <c r="A7" s="24"/>
+      <c r="B7" s="18"/>
       <c r="C7" s="25"/>
       <c r="D7" s="1" t="s">
         <v>46</v>
@@ -6118,8 +5838,8 @@
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A8" s="20"/>
-      <c r="B8" s="22"/>
+      <c r="A8" s="24"/>
+      <c r="B8" s="18"/>
       <c r="C8" s="25"/>
       <c r="D8" s="1" t="s">
         <v>47</v>
@@ -6141,10 +5861,10 @@
       </c>
     </row>
     <row r="10" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="24" t="s">
         <v>185</v>
       </c>
-      <c r="B10" s="22" t="s">
+      <c r="B10" s="18" t="s">
         <v>50</v>
       </c>
       <c r="C10" s="25" t="s">
@@ -6170,8 +5890,8 @@
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A11" s="20"/>
-      <c r="B11" s="22"/>
+      <c r="A11" s="24"/>
+      <c r="B11" s="18"/>
       <c r="C11" s="25"/>
       <c r="D11" s="1" t="s">
         <v>46</v>
@@ -6193,8 +5913,8 @@
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A12" s="20"/>
-      <c r="B12" s="22"/>
+      <c r="A12" s="24"/>
+      <c r="B12" s="18"/>
       <c r="C12" s="25"/>
       <c r="D12" s="1" t="s">
         <v>47</v>
@@ -6213,10 +5933,10 @@
       </c>
     </row>
     <row r="14" spans="1:9" s="3" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="20" t="s">
+      <c r="A14" s="24" t="s">
         <v>184</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="18" t="s">
         <v>51</v>
       </c>
       <c r="C14" s="25" t="s">
@@ -6242,8 +5962,8 @@
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A15" s="20"/>
-      <c r="B15" s="22"/>
+      <c r="A15" s="24"/>
+      <c r="B15" s="18"/>
       <c r="C15" s="25"/>
       <c r="D15" s="1" t="s">
         <v>46</v>
@@ -6265,8 +5985,8 @@
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A16" s="20"/>
-      <c r="B16" s="22"/>
+      <c r="A16" s="24"/>
+      <c r="B16" s="18"/>
       <c r="C16" s="25"/>
       <c r="D16" s="1" t="s">
         <v>47</v>
@@ -6288,10 +6008,10 @@
       </c>
     </row>
     <row r="18" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="20" t="s">
+      <c r="A18" s="24" t="s">
         <v>183</v>
       </c>
-      <c r="B18" s="22" t="s">
+      <c r="B18" s="18" t="s">
         <v>52</v>
       </c>
       <c r="C18" s="25" t="s">
@@ -6317,8 +6037,8 @@
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A19" s="20"/>
-      <c r="B19" s="22"/>
+      <c r="A19" s="24"/>
+      <c r="B19" s="18"/>
       <c r="C19" s="25"/>
       <c r="D19" s="1" t="s">
         <v>46</v>
@@ -6340,8 +6060,8 @@
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A20" s="20"/>
-      <c r="B20" s="22"/>
+      <c r="A20" s="24"/>
+      <c r="B20" s="18"/>
       <c r="C20" s="25"/>
       <c r="D20" s="1" t="s">
         <v>47</v>
@@ -6360,10 +6080,10 @@
       </c>
     </row>
     <row r="22" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="20" t="s">
+      <c r="A22" s="24" t="s">
         <v>181</v>
       </c>
-      <c r="B22" s="22" t="s">
+      <c r="B22" s="18" t="s">
         <v>53</v>
       </c>
       <c r="C22" s="25" t="s">
@@ -6389,8 +6109,8 @@
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A23" s="20"/>
-      <c r="B23" s="22"/>
+      <c r="A23" s="24"/>
+      <c r="B23" s="18"/>
       <c r="C23" s="25"/>
       <c r="D23" s="1" t="s">
         <v>46</v>
@@ -6412,8 +6132,8 @@
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A24" s="20"/>
-      <c r="B24" s="22"/>
+      <c r="A24" s="24"/>
+      <c r="B24" s="18"/>
       <c r="C24" s="25"/>
       <c r="D24" s="1" t="s">
         <v>47</v>
@@ -6589,7 +6309,7 @@
       </c>
     </row>
     <row r="34" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="20" t="s">
+      <c r="A34" s="24" t="s">
         <v>179</v>
       </c>
       <c r="B34" s="25" t="s">
@@ -6618,7 +6338,7 @@
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A35" s="20"/>
+      <c r="A35" s="24"/>
       <c r="B35" s="25"/>
       <c r="C35" s="25"/>
       <c r="D35" s="1" t="s">
@@ -6641,7 +6361,7 @@
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A36" s="20"/>
+      <c r="A36" s="24"/>
       <c r="B36" s="25"/>
       <c r="C36" s="25"/>
       <c r="D36" s="1" t="s">
@@ -6664,10 +6384,10 @@
       </c>
     </row>
     <row r="38" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="20" t="s">
+      <c r="A38" s="24" t="s">
         <v>182</v>
       </c>
-      <c r="B38" s="20" t="s">
+      <c r="B38" s="24" t="s">
         <v>177</v>
       </c>
       <c r="C38" s="25" t="s">
@@ -6678,26 +6398,26 @@
       </c>
     </row>
     <row r="39" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="20"/>
-      <c r="B39" s="20"/>
+      <c r="A39" s="24"/>
+      <c r="B39" s="24"/>
       <c r="C39" s="25"/>
       <c r="D39" s="1" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="20"/>
-      <c r="B40" s="20"/>
+      <c r="A40" s="24"/>
+      <c r="B40" s="24"/>
       <c r="C40" s="25"/>
       <c r="D40" s="1" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="42" spans="1:9" s="3" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="20" t="s">
+      <c r="A42" s="24" t="s">
         <v>188</v>
       </c>
-      <c r="B42" s="20" t="s">
+      <c r="B42" s="24" t="s">
         <v>189</v>
       </c>
       <c r="C42" s="25" t="s">
@@ -6723,8 +6443,8 @@
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A43" s="20"/>
-      <c r="B43" s="20"/>
+      <c r="A43" s="24"/>
+      <c r="B43" s="24"/>
       <c r="C43" s="25"/>
       <c r="D43" s="1" t="s">
         <v>46</v>
@@ -6746,8 +6466,8 @@
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A44" s="20"/>
-      <c r="B44" s="20"/>
+      <c r="A44" s="24"/>
+      <c r="B44" s="24"/>
       <c r="C44" s="25"/>
       <c r="D44" s="1" t="s">
         <v>47</v>
@@ -6769,10 +6489,10 @@
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A46" s="20" t="s">
+      <c r="A46" s="24" t="s">
         <v>191</v>
       </c>
-      <c r="B46" s="20" t="s">
+      <c r="B46" s="24" t="s">
         <v>194</v>
       </c>
       <c r="C46" s="25" t="s">
@@ -6798,8 +6518,8 @@
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A47" s="20"/>
-      <c r="B47" s="20"/>
+      <c r="A47" s="24"/>
+      <c r="B47" s="24"/>
       <c r="C47" s="25"/>
       <c r="D47" s="1" t="s">
         <v>46</v>
@@ -6821,8 +6541,8 @@
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A48" s="20"/>
-      <c r="B48" s="20"/>
+      <c r="A48" s="24"/>
+      <c r="B48" s="24"/>
       <c r="C48" s="25"/>
       <c r="D48" s="1" t="s">
         <v>47</v>
@@ -6845,28 +6565,6 @@
     </row>
   </sheetData>
   <mergeCells count="36">
-    <mergeCell ref="A46:A48"/>
-    <mergeCell ref="B46:B48"/>
-    <mergeCell ref="C46:C48"/>
-    <mergeCell ref="A30:A32"/>
-    <mergeCell ref="B30:B32"/>
-    <mergeCell ref="C30:C32"/>
-    <mergeCell ref="A38:A40"/>
-    <mergeCell ref="B38:B40"/>
-    <mergeCell ref="C38:C40"/>
-    <mergeCell ref="A42:A44"/>
-    <mergeCell ref="B42:B44"/>
-    <mergeCell ref="C42:C44"/>
-    <mergeCell ref="C34:C36"/>
-    <mergeCell ref="A6:A8"/>
-    <mergeCell ref="A34:A36"/>
-    <mergeCell ref="B34:B36"/>
-    <mergeCell ref="A26:A28"/>
-    <mergeCell ref="A2:A4"/>
-    <mergeCell ref="A10:A12"/>
-    <mergeCell ref="A14:A16"/>
-    <mergeCell ref="A18:A20"/>
-    <mergeCell ref="A22:A24"/>
     <mergeCell ref="C22:C24"/>
     <mergeCell ref="C26:C28"/>
     <mergeCell ref="B26:B28"/>
@@ -6881,6 +6579,28 @@
     <mergeCell ref="C18:C20"/>
     <mergeCell ref="B18:B20"/>
     <mergeCell ref="B22:B24"/>
+    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="A34:A36"/>
+    <mergeCell ref="B34:B36"/>
+    <mergeCell ref="A26:A28"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="A18:A20"/>
+    <mergeCell ref="A22:A24"/>
+    <mergeCell ref="A46:A48"/>
+    <mergeCell ref="B46:B48"/>
+    <mergeCell ref="C46:C48"/>
+    <mergeCell ref="A30:A32"/>
+    <mergeCell ref="B30:B32"/>
+    <mergeCell ref="C30:C32"/>
+    <mergeCell ref="A38:A40"/>
+    <mergeCell ref="B38:B40"/>
+    <mergeCell ref="C38:C40"/>
+    <mergeCell ref="A42:A44"/>
+    <mergeCell ref="B42:B44"/>
+    <mergeCell ref="C42:C44"/>
+    <mergeCell ref="C34:C36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>